<commit_message>
Develop source atlas, challenge records, chronology comparison and book-museum handoff
</commit_message>
<xml_diff>
--- a/theology-wiki/planning/Theology-Research-Plan.xlsx
+++ b/theology-wiki/planning/Theology-Research-Plan.xlsx
@@ -2,15 +2,15 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="1" r:id="Rbe3742539e514d2d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Checklist" sheetId="2" r:id="R877be50122474d54"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dependencies" sheetId="3" r:id="R01d8e424d1a94b00"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Chapter Map" sheetId="4" r:id="R1c91f99d94c74608"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Source Coverage" sheetId="5" r:id="R69cf1173c3394fdb"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Textual Evidence" sheetId="6" r:id="R961e3b9b2e2f40b3"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Intellectual Debts" sheetId="7" r:id="Recf913cc26eb4e82"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Release Gates" sheetId="8" r:id="Rce7c006f21fd4e22"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Read Me" sheetId="9" r:id="R711a937ffa314231"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="1" r:id="Rcb2262bbb8624441"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Checklist" sheetId="2" r:id="R918f795bc6354fd3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dependencies" sheetId="3" r:id="R7d755c68f9e6430f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Chapter Map" sheetId="4" r:id="R46e098001a824931"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Source Coverage" sheetId="5" r:id="R51cacab203544372"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Textual Evidence" sheetId="6" r:id="R160766a8037e4e72"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Intellectual Debts" sheetId="7" r:id="R57bd662050164277"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Release Gates" sheetId="8" r:id="R01a51663494f4067"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Read Me" sheetId="9" r:id="R4f2a5533abdb416b"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -259,14 +259,14 @@
         <x:color rgb="FF23573B"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFDCEFE6"/>
         </x:patternFill>
       </x:fill>
     </x:dxf>
     <x:dxf>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFBE4DC"/>
         </x:patternFill>
       </x:fill>
@@ -429,7 +429,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Rc60b286167674bfe"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R80ac55a97be047fc"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -841,7 +841,7 @@
     </x:row>
     <x:row r="5">
       <x:c r="A5" s="36" t="str">
-        <x:v>Shared snapshot: 2026.09.05-roadmap-1</x:v>
+        <x:v>Shared snapshot: 2026.09.05-atlas-1</x:v>
       </x:c>
       <x:c r="B5" s="36"/>
       <x:c r="C5" s="36"/>
@@ -908,7 +908,7 @@
       <x:c r="F8" s="60"/>
       <x:c r="G8" s="60" t="n">
         <x:f>COUNTIF(Checklist!P7:P42,"Ready")</x:f>
-        <x:v>9</x:v>
+        <x:v>7</x:v>
       </x:c>
       <x:c r="H8" s="60"/>
       <x:c r="I8" s="60"/>
@@ -1222,7 +1222,7 @@
       <x:c r="E25" s="36"/>
       <x:c r="F25" s="36" t="n">
         <x:f>COUNTIF('Source Coverage'!H7:H360,"&gt;0")</x:f>
-        <x:v>11</x:v>
+        <x:v>13</x:v>
       </x:c>
       <x:c r="G25" s="36"/>
       <x:c r="H25" s="36"/>
@@ -1266,7 +1266,7 @@
     </x:row>
     <x:row r="28" ht="23" customHeight="1">
       <x:c r="A28" s="54" t="str">
-        <x:v>NEXT SUBSTANTIVE WORK: verify the critical 11Q13 and printed Nag Hammadi editions, extend the Thomas comparison, locate precise Tabor citations, and test the proposed historical carriers. The first Melchizedek comparison is a delivered pass, not closure of that larger investigation.</x:v>
+        <x:v>NEW FOUNDATION: a typed source atlas, six auditable chronology intervals, four recovered challenge records and three content-only museum trails. The expanded Exodus and transmission studies support existing book routes. Historical-carrier and critical-edition tasks remain open.</x:v>
       </x:c>
       <x:c r="B28" s="54"/>
       <x:c r="C28" s="54"/>
@@ -1410,7 +1410,7 @@
     <x:mergeCell ref="A32:L33"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R49061f94d0334211"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R77b532c5011d4a47"/>
 </x:worksheet>
 </file>
 
@@ -1514,7 +1514,7 @@
     </x:row>
     <x:row r="5" ht="20" customHeight="1">
       <x:c r="A5" s="14" t="str">
-        <x:v>Snapshot 2026-09-05 | 2026.09.05-roadmap-1 | Shared plan: theology-wiki/editorial/roadmap.json</x:v>
+        <x:v>Snapshot 2026-09-05 | 2026.09.05-atlas-1 | Shared plan: theology-wiki/editorial/roadmap.json</x:v>
       </x:c>
       <x:c r="B5" s="14"/>
       <x:c r="C5" s="14"/>
@@ -2153,7 +2153,7 @@
         <x:v>P1</x:v>
       </x:c>
       <x:c r="E19" s="28" t="str">
-        <x:v>Not started</x:v>
+        <x:v>Draft</x:v>
       </x:c>
       <x:c r="F19" s="28" t="str">
         <x:v>Editorial/research work (unassigned)</x:v>
@@ -2166,9 +2166,11 @@
         <x:v>Prerequisites met</x:v>
       </x:c>
       <x:c r="I19" s="23" t="str">
-        <x:v>Distinguish preservation in a region, movement of texts and biological or institutional lineage. Attach evidence to each proposed bridge.</x:v>
-      </x:c>
-      <x:c r="J19" s="23" t="str"/>
+        <x:v>Distinguish preservation in a region, movement of texts and biological or institutional lineage. Attach evidence to each proposed bridge. The first reception comparison is available, but the proposed institutional carriers and exact critical editions remain to be tested.</x:v>
+      </x:c>
+      <x:c r="J19" s="23" t="str">
+        <x:v>theology-wiki/content/developed/manuscripts-movements-and-survival.md</x:v>
+      </x:c>
       <x:c r="K19" s="30"/>
       <x:c r="L19" s="28" t="str"/>
       <x:c r="M19" s="23" t="str">
@@ -2183,7 +2185,6 @@
       </x:c>
       <x:c r="P19" s="23" t="str">
         <x:f>IF(AND(E19="Not started",H19="Prerequisites met"),"Ready","")</x:f>
-        <x:v>Ready</x:v>
       </x:c>
     </x:row>
     <x:row r="20" ht="94" customHeight="1">
@@ -2731,7 +2732,7 @@
         <x:v>P0</x:v>
       </x:c>
       <x:c r="E31" s="28" t="str">
-        <x:v>Not started</x:v>
+        <x:v>Draft</x:v>
       </x:c>
       <x:c r="F31" s="28" t="str">
         <x:v>Editorial/research work (unassigned)</x:v>
@@ -2745,9 +2746,12 @@
         <x:v>Prerequisites met</x:v>
       </x:c>
       <x:c r="I31" s="23" t="str">
-        <x:v>Every developed article has reviewed claims, original corrections, rejected readings and a scoped list of sources; source linking alone is not a fidelity sign-off.</x:v>
-      </x:c>
-      <x:c r="J31" s="23" t="str"/>
+        <x:v>Every developed article has reviewed claims, original corrections, rejected readings and a scoped list of sources; source linking alone is not a fidelity sign-off. The first source-atlas pass adds four explicitly bounded challenge records; remaining article dossiers and author review are still required.</x:v>
+      </x:c>
+      <x:c r="J31" s="23" t="str">
+        <x:v>theology-wiki/data/source-atlas.json
+theology-wiki/content/developed/exodus-to-temple-competing-chronologies.md</x:v>
+      </x:c>
       <x:c r="K31" s="30"/>
       <x:c r="L31" s="28" t="str"/>
       <x:c r="M31" s="23" t="str"/>
@@ -2760,7 +2764,6 @@
       </x:c>
       <x:c r="P31" s="23" t="str">
         <x:f>IF(AND(E31="Not started",H31="Prerequisites met"),"Ready","")</x:f>
-        <x:v>Ready</x:v>
       </x:c>
     </x:row>
     <x:row r="32" ht="94" customHeight="1">
@@ -3307,7 +3310,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rabac885b5a044822"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7d77b65399f14863"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3362,7 +3365,7 @@
     </x:row>
     <x:row r="5" ht="20" customHeight="1">
       <x:c r="A5" s="14" t="str">
-        <x:v>Snapshot 2026-09-05 | 2026.09.05-roadmap-1 | Shared plan: theology-wiki/editorial/roadmap.json</x:v>
+        <x:v>Snapshot 2026-09-05 | 2026.09.05-atlas-1 | Shared plan: theology-wiki/editorial/roadmap.json</x:v>
       </x:c>
       <x:c r="B5" s="14"/>
       <x:c r="C5" s="14"/>
@@ -4040,7 +4043,7 @@
       </x:c>
       <x:c r="D36" s="23" t="str">
         <x:f>IFERROR(INDEX(Checklist!$E$7:$E$42,MATCH(B36,Checklist!$A$7:$A$42,0)),"Unknown ID")</x:f>
-        <x:v>Not started</x:v>
+        <x:v>Draft</x:v>
       </x:c>
       <x:c r="E36" s="23" t="n">
         <x:f>IF(D36="Verified output",1,0)</x:f>
@@ -4366,7 +4369,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6500d7f601bd4f3c"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R09a8ae9aaeed4b6c"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4446,7 +4449,7 @@
     </x:row>
     <x:row r="5" ht="20" customHeight="1">
       <x:c r="A5" s="14" t="str">
-        <x:v>Snapshot 2026-09-05 | 2026.09.05-roadmap-1 | Shared plan: theology-wiki/editorial/roadmap.json</x:v>
+        <x:v>Snapshot 2026-09-05 | 2026.09.05-atlas-1 | Shared plan: theology-wiki/editorial/roadmap.json</x:v>
       </x:c>
       <x:c r="B5" s="14"/>
       <x:c r="C5" s="14"/>
@@ -4594,15 +4597,17 @@
         <x:v>Not assessed as a manuscript chapter</x:v>
       </x:c>
       <x:c r="E9" s="23" t="str">
-        <x:v>moses-volcano-and-exodus-chronology</x:v>
+        <x:v>moses-volcano-and-exodus-chronology
+exodus-to-temple-competing-chronologies</x:v>
       </x:c>
       <x:c r="F9" s="23" t="str">
         <x:v>moses-dating-debate
-parthians-and-medes-meaning</x:v>
+parthians-and-medes-meaning
+daniel-and-teacher-of-righteousness</x:v>
       </x:c>
       <x:c r="G9" s="23" t="n">
         <x:f>IF(F9="",0,LEN(F9)-LEN(SUBSTITUTE(F9,CHAR(10),""))+1)</x:f>
-        <x:v>2</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="H9" s="23" t="str">
         <x:v>chapter-arc
@@ -4675,7 +4680,8 @@
       </x:c>
       <x:c r="E11" s="23" t="str">
         <x:v>tor-thomas-and-gnostic-transmission
-melchizedek-priesthood-and-transmission</x:v>
+melchizedek-priesthood-and-transmission
+manuscripts-movements-and-survival</x:v>
       </x:c>
       <x:c r="F11" s="23" t="str">
         <x:v>teacher-of-righteousness-vs-gnostic-jesus
@@ -5223,7 +5229,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rcb49a45c31e24f1a"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb0801acb58214264"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5318,7 +5324,7 @@
     </x:row>
     <x:row r="5" ht="20" customHeight="1">
       <x:c r="A5" s="14" t="str">
-        <x:v>Snapshot 2026-09-05 | 2026.09.05-roadmap-1 | Shared plan: theology-wiki/editorial/roadmap.json</x:v>
+        <x:v>Snapshot 2026-09-05 | 2026.09.05-atlas-1 | Shared plan: theology-wiki/editorial/roadmap.json</x:v>
       </x:c>
       <x:c r="B5" s="14"/>
       <x:c r="C5" s="14"/>
@@ -5771,14 +5777,16 @@
         <x:v>jesus-teacher-of-righteousness-hypothesis
 sacred-inheritance-and-rival-continuations
 tor-thomas-and-gnostic-transmission
-melchizedek-priesthood-and-transmission</x:v>
+melchizedek-priesthood-and-transmission
+manuscripts-movements-and-survival</x:v>
       </x:c>
       <x:c r="F16" s="23" t="n">
         <x:f>IF(E16="",0,LEN(E16)-LEN(SUBSTITUTE(E16,CHAR(10),""))+1)</x:f>
-        <x:v>4</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="G16" s="23" t="str">
-        <x:v>Turn 24
+        <x:v>Turn 22
+Turn 24
 Turn 26
 Turn 63
 Turn 82
@@ -5786,7 +5794,7 @@
       </x:c>
       <x:c r="H16" s="23" t="n">
         <x:f>IF(G16="",0,LEN(G16&amp;"")-LEN(SUBSTITUTE(G16&amp;"",CHAR(10),""))+1)</x:f>
-        <x:v>5</x:v>
+        <x:v>6</x:v>
       </x:c>
       <x:c r="I16" s="23" t="str">
         <x:v>shared-archive
@@ -8892,11 +8900,12 @@
       </x:c>
       <x:c r="E93" s="23" t="str">
         <x:v>jesus-teacher-of-righteousness-hypothesis
-tor-thomas-and-gnostic-transmission</x:v>
+tor-thomas-and-gnostic-transmission
+exodus-to-temple-competing-chronologies</x:v>
       </x:c>
       <x:c r="F93" s="23" t="n">
         <x:f>IF(E93="",0,LEN(E93)-LEN(SUBSTITUTE(E93,CHAR(10),""))+1)</x:f>
-        <x:v>2</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="G93" s="23" t="str"/>
       <x:c r="H93" s="23" t="n">
@@ -8904,7 +8913,8 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="I93" s="23" t="str">
-        <x:v>teacher-identity
+        <x:v>catastrophe-memory
+teacher-identity
 thomas</x:v>
       </x:c>
       <x:c r="J93" s="23" t="str">
@@ -13538,16 +13548,19 @@
       <x:c r="E208" s="23" t="str">
         <x:v>apocalyptic-repair-theology
 gnosticism-and-temple-trauma
-tor-thomas-and-gnostic-transmission</x:v>
+tor-thomas-and-gnostic-transmission
+manuscripts-movements-and-survival</x:v>
       </x:c>
       <x:c r="F208" s="23" t="n">
         <x:f>IF(E208="",0,LEN(E208)-LEN(SUBSTITUTE(E208,CHAR(10),""))+1)</x:f>
-        <x:v>3</x:v>
-      </x:c>
-      <x:c r="G208" s="23" t="str"/>
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="G208" s="23" t="str">
+        <x:v>Turn 1</x:v>
+      </x:c>
       <x:c r="H208" s="23" t="n">
         <x:f>IF(G208="",0,LEN(G208&amp;"")-LEN(SUBSTITUTE(G208&amp;"",CHAR(10),""))+1)</x:f>
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="I208" s="23" t="str">
         <x:v>thomas
@@ -15361,16 +15374,21 @@
         <x:v>62</x:v>
       </x:c>
       <x:c r="E253" s="23" t="str">
-        <x:v>moses-volcano-and-exodus-chronology</x:v>
+        <x:v>moses-volcano-and-exodus-chronology
+exodus-to-temple-competing-chronologies</x:v>
       </x:c>
       <x:c r="F253" s="23" t="n">
         <x:f>IF(E253="",0,LEN(E253)-LEN(SUBSTITUTE(E253,CHAR(10),""))+1)</x:f>
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="G253" s="23" t="str"/>
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="G253" s="23" t="str">
+        <x:v>Turn 23
+Turn 29
+Turn 46</x:v>
+      </x:c>
       <x:c r="H253" s="23" t="n">
         <x:f>IF(G253="",0,LEN(G253&amp;"")-LEN(SUBSTITUTE(G253&amp;"",CHAR(10),""))+1)</x:f>
-        <x:v>0</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="I253" s="23" t="str">
         <x:v>catastrophe-memory</x:v>
@@ -19759,7 +19777,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R843d0fce597f4995"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R93dd8d4df2df4e3f"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -19824,7 +19842,7 @@
     </x:row>
     <x:row r="5" ht="20" customHeight="1">
       <x:c r="A5" s="14" t="str">
-        <x:v>Snapshot 2026-09-05 | 2026.09.05-roadmap-1 | Shared plan: theology-wiki/editorial/roadmap.json</x:v>
+        <x:v>Snapshot 2026-09-05 | 2026.09.05-atlas-1 | Shared plan: theology-wiki/editorial/roadmap.json</x:v>
       </x:c>
       <x:c r="B5" s="14"/>
       <x:c r="C5" s="14"/>
@@ -19998,7 +20016,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4b8c2230c37c46ee"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re0af85e12088448c"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -20053,7 +20071,7 @@
     </x:row>
     <x:row r="5" ht="20" customHeight="1">
       <x:c r="A5" s="14" t="str">
-        <x:v>Snapshot 2026-09-05 | 2026.09.05-roadmap-1 | Shared plan: theology-wiki/editorial/roadmap.json</x:v>
+        <x:v>Snapshot 2026-09-05 | 2026.09.05-atlas-1 | Shared plan: theology-wiki/editorial/roadmap.json</x:v>
       </x:c>
       <x:c r="B5" s="14"/>
       <x:c r="C5" s="14"/>
@@ -20203,7 +20221,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R78a9269ba7434a98"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R96d951f3b94d4013"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -20253,7 +20271,7 @@
     </x:row>
     <x:row r="5" ht="20" customHeight="1">
       <x:c r="A5" s="14" t="str">
-        <x:v>Snapshot 2026-09-05 | 2026.09.05-roadmap-1 | Shared plan: theology-wiki/editorial/roadmap.json</x:v>
+        <x:v>Snapshot 2026-09-05 | 2026.09.05-atlas-1 | Shared plan: theology-wiki/editorial/roadmap.json</x:v>
       </x:c>
       <x:c r="B5" s="14"/>
       <x:c r="C5" s="14"/>
@@ -20409,7 +20427,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc6b1251d25a5488f"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb4223a544f0149c2"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -20444,7 +20462,7 @@
     </x:row>
     <x:row r="5" ht="20" customHeight="1">
       <x:c r="A5" s="14" t="str">
-        <x:v>Snapshot 2026-09-05 | 2026.09.05-roadmap-1 | Shared plan: theology-wiki/editorial/roadmap.json</x:v>
+        <x:v>Snapshot 2026-09-05 | 2026.09.05-atlas-1 | Shared plan: theology-wiki/editorial/roadmap.json</x:v>
       </x:c>
       <x:c r="B5" s="14"/>
     </x:row>
@@ -20549,7 +20567,7 @@
         <x:v>Next writing pass</x:v>
       </x:c>
       <x:c r="B18" s="23" t="str">
-        <x:v>Use the ready-to-start filter, finish a bounded comparison, retain author qualifications, update evidence and the shared task, then regenerate coverage.</x:v>
+        <x:v>The source atlas adds typed records, exact challenge passages and content-only museum trails. Follow its remaining questions into the shared roadmap; no label replaces the full argument.</x:v>
       </x:c>
     </x:row>
     <x:row r="19" ht="64" customHeight="1">
@@ -20573,7 +20591,7 @@
         <x:v>Snapshot version</x:v>
       </x:c>
       <x:c r="B21" s="23" t="str">
-        <x:v>2026.09.05-roadmap-1</x:v>
+        <x:v>2026.09.05-atlas-1</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -20584,7 +20602,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R93a92c4e8a844af9"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8ff5d24a82ad47f6"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Implement authorial Theology articles, Christic formation research and museum trail
</commit_message>
<xml_diff>
--- a/theology-wiki/planning/Theology-Research-Plan.xlsx
+++ b/theology-wiki/planning/Theology-Research-Plan.xlsx
@@ -2,15 +2,15 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="1" r:id="Rcb2262bbb8624441"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Checklist" sheetId="2" r:id="R918f795bc6354fd3"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dependencies" sheetId="3" r:id="R7d755c68f9e6430f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Chapter Map" sheetId="4" r:id="R46e098001a824931"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Source Coverage" sheetId="5" r:id="R51cacab203544372"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Textual Evidence" sheetId="6" r:id="R160766a8037e4e72"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Intellectual Debts" sheetId="7" r:id="R57bd662050164277"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Release Gates" sheetId="8" r:id="R01a51663494f4067"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Read Me" sheetId="9" r:id="R4f2a5533abdb416b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="1" r:id="R6ea75ee899904e79"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Checklist" sheetId="2" r:id="R2095133822714301"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dependencies" sheetId="3" r:id="Ra2546f1206804a0b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Chapter Map" sheetId="4" r:id="R9898f80c5b954c18"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Source Coverage" sheetId="5" r:id="Rc99b733cbee54933"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Textual Evidence" sheetId="6" r:id="R4fdd83ac3d484699"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Intellectual Debts" sheetId="7" r:id="R10ede73d3d474e16"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Release Gates" sheetId="8" r:id="Rd4053f7b59e94f01"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Read Me" sheetId="9" r:id="Re06f9aaadd174dd9"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -429,7 +429,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R80ac55a97be047fc"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Rd1fac09bf3f745d2"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -1410,7 +1410,7 @@
     <x:mergeCell ref="A32:L33"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R77b532c5011d4a47"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0ede1000e6f64752"/>
 </x:worksheet>
 </file>
 
@@ -3310,7 +3310,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7d77b65399f14863"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7e6fcd7818ef4804"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4369,7 +4369,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R09a8ae9aaeed4b6c"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7678d0f99d4642bc"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4845,14 +4845,15 @@
         <x:v>The inheritance inside a mind</x:v>
       </x:c>
       <x:c r="C15" s="23" t="str">
-        <x:v>Christ as an active moral model</x:v>
+        <x:v>Christic self-formation and bounded agency</x:v>
       </x:c>
       <x:c r="D15" s="23" t="str">
         <x:v>Not assessed as a manuscript chapter</x:v>
       </x:c>
       <x:c r="E15" s="23" t="str">
         <x:v>christ-as-an-inner-model
-divine-will-and-self-authorizing-power</x:v>
+divine-will-and-self-authorizing-power
+inner-formation-texts-and-material-witnesses</x:v>
       </x:c>
       <x:c r="F15" s="23" t="str">
         <x:v>cognitive-gnosticism-jesus-vs-gnostic-jesus
@@ -4860,11 +4861,12 @@
 teacher-of-righteousness-vs-gnostic-jesus
 samuel-vs-micah-divide
 resurrection-debate-in-christianity
-agi-religious-framework</x:v>
+agi-religious-framework
+ai-re-dates-dead-sea-scrolls</x:v>
       </x:c>
       <x:c r="G15" s="23" t="n">
         <x:f>IF(F15="",0,LEN(F15)-LEN(SUBSTITUTE(F15,CHAR(10),""))+1)</x:f>
-        <x:v>6</x:v>
+        <x:v>7</x:v>
       </x:c>
       <x:c r="H15" s="23" t="str">
         <x:v>will
@@ -4876,7 +4878,7 @@
         <x:v>Not reviewed</x:v>
       </x:c>
       <x:c r="J15" s="23" t="str">
-        <x:v>Follow the comparison, the changed action and the subsequent correction of the model.</x:v>
+        <x:v>Develop the embodied self, learned self-model, recurrent choice and correction of the Christ model, then examine the textual and material history of formation.</x:v>
       </x:c>
       <x:c r="K15" s="23" t="str">
         <x:v>https://v5ma.github.io/theology-wiki/san-reader.html?page=book-contents#chapter-inner-model</x:v>
@@ -5229,7 +5231,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb0801acb58214264"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4d78b3ea18a242f3"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5778,11 +5780,12 @@
 sacred-inheritance-and-rival-continuations
 tor-thomas-and-gnostic-transmission
 melchizedek-priesthood-and-transmission
-manuscripts-movements-and-survival</x:v>
+manuscripts-movements-and-survival
+inner-formation-texts-and-material-witnesses</x:v>
       </x:c>
       <x:c r="F16" s="23" t="n">
         <x:f>IF(E16="",0,LEN(E16)-LEN(SUBSTITUTE(E16,CHAR(10),""))+1)</x:f>
-        <x:v>5</x:v>
+        <x:v>6</x:v>
       </x:c>
       <x:c r="G16" s="23" t="str">
         <x:v>Turn 22
@@ -5800,6 +5803,7 @@
         <x:v>shared-archive
 teacher-identity
 thomas
+inner-model
 continuing</x:v>
       </x:c>
       <x:c r="J16" s="23" t="str">
@@ -8647,11 +8651,12 @@
 religion-for-conscious-robots
 divine-will-and-self-authorizing-power
 scripture-power-and-repair
-god-and-our-models-of-god</x:v>
+god-and-our-models-of-god
+inner-formation-texts-and-material-witnesses</x:v>
       </x:c>
       <x:c r="F87" s="23" t="n">
         <x:f>IF(E87="",0,LEN(E87)-LEN(SUBSTITUTE(E87,CHAR(10),""))+1)</x:f>
-        <x:v>6</x:v>
+        <x:v>7</x:v>
       </x:c>
       <x:c r="G87" s="23" t="str">
         <x:v>Turn 23</x:v>
@@ -19777,7 +19782,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R93dd8d4df2df4e3f"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rff190be5c8704059"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -20016,7 +20021,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re0af85e12088448c"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R59d4f2f71d95422d"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -20128,7 +20133,7 @@
         <x:v>Aaron Abke and Abraham Hicks</x:v>
       </x:c>
       <x:c r="B8" s="23" t="str">
-        <x:v>Teachers discussed by the author</x:v>
+        <x:v>Teachers discussed in the source inquiry</x:v>
       </x:c>
       <x:c r="C8" s="23" t="str">
         <x:v>Comparisons involving faith, inward experience, spiritual vocabulary and the relation of different traditions.</x:v>
@@ -20152,7 +20157,7 @@
         <x:v>Translation of Thomas used for the present passage comparisons.</x:v>
       </x:c>
       <x:c r="D9" s="23" t="str">
-        <x:v>This credit records the edition's textual source. It does not retrospectively identify these translators as the author's personal influences.</x:v>
+        <x:v>This credit records the edition's textual source. It does not retrospectively identify these translators as my personal influences.</x:v>
       </x:c>
       <x:c r="E9" s="23" t="str"/>
       <x:c r="F9" s="23" t="str">
@@ -20221,7 +20226,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R96d951f3b94d4013"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7a685de753c8446b"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -20371,7 +20376,7 @@
         <x:v>Authorial review</x:v>
       </x:c>
       <x:c r="C11" s="23" t="str">
-        <x:v>Micah approves the actual chapter wording and the treatment of his arguments.</x:v>
+        <x:v>I approve the actual chapter wording and the treatment of the arguments.</x:v>
       </x:c>
       <x:c r="D11" s="23" t="str">
         <x:v>Not assessed</x:v>
@@ -20427,7 +20432,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb4223a544f0149c2"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re902cc0244bd4962"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -20588,10 +20593,10 @@
     </x:row>
     <x:row r="21" ht="64" customHeight="1">
       <x:c r="A21" s="23" t="str">
-        <x:v>Snapshot version</x:v>
+        <x:v>Authorial text refresh</x:v>
       </x:c>
       <x:c r="B21" s="23" t="str">
-        <x:v>2026.09.05-atlas-1</x:v>
+        <x:v>2026-09-06. Chapter and source links reflect the Christic Self-Formation working edition. Shared task statuses remain unchanged.</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -20602,7 +20607,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8ff5d24a82ad47f6"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9c31d36598f143cc"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Integrate authorial Theology, computational argument map and flood-inheritance research
</commit_message>
<xml_diff>
--- a/theology-wiki/planning/Theology-Research-Plan.xlsx
+++ b/theology-wiki/planning/Theology-Research-Plan.xlsx
@@ -2,15 +2,15 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="1" r:id="Rcb2262bbb8624441"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Checklist" sheetId="2" r:id="R918f795bc6354fd3"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dependencies" sheetId="3" r:id="R7d755c68f9e6430f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Chapter Map" sheetId="4" r:id="R46e098001a824931"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Source Coverage" sheetId="5" r:id="R51cacab203544372"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Textual Evidence" sheetId="6" r:id="R160766a8037e4e72"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Intellectual Debts" sheetId="7" r:id="R57bd662050164277"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Release Gates" sheetId="8" r:id="R01a51663494f4067"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Read Me" sheetId="9" r:id="R4f2a5533abdb416b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="1" r:id="Re2d3d0ccd1aa42cb"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Checklist" sheetId="2" r:id="R2a390d67b28046d7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dependencies" sheetId="3" r:id="R79b095d7815e462a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Chapter Map" sheetId="4" r:id="Rbca6cae0a1904265"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Source Coverage" sheetId="5" r:id="Rb07684c45cd54ea9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Textual Evidence" sheetId="6" r:id="R4184e020bbb24bb6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Intellectual Debts" sheetId="7" r:id="R0fe8fc9b8df046db"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Release Gates" sheetId="8" r:id="R68f57a01693c432a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Read Me" sheetId="9" r:id="Rf45f6f597ad740a3"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -25,7 +25,7 @@
     <x:numFmt numFmtId="200" formatCode="yyyy-mm-dd"/>
     <x:numFmt numFmtId="201" formatCode="#,##0"/>
   </x:numFmts>
-  <x:fonts count="12">
+  <x:fonts count="13">
     <x:font>
       <x:sz val="11"/>
       <x:name val="Carlito"/>
@@ -91,6 +91,11 @@
       <x:color rgb="FFFFFFFF"/>
       <x:name val="Aptos"/>
     </x:font>
+    <x:font>
+      <x:sz val="9"/>
+      <x:color rgb="FF203543"/>
+      <x:name val="Aptos"/>
+    </x:font>
   </x:fonts>
   <x:fills count="5">
     <x:fill>
@@ -122,7 +127,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="62">
+  <x:cellXfs count="65">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -248,6 +253,11 @@
     </x:xf>
     <x:xf numFmtId="0" fontId="10" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
     </x:xf>
   </x:cellXfs>
   <x:cellStyles count="1">
@@ -429,7 +439,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R80ac55a97be047fc"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R227952ecf9ee446a"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -839,15 +849,15 @@
       <x:c r="K4" s="36"/>
       <x:c r="L4" s="36"/>
     </x:row>
-    <x:row r="5">
-      <x:c r="A5" s="36" t="str">
-        <x:v>Shared snapshot: 2026.09.05-atlas-1</x:v>
-      </x:c>
-      <x:c r="B5" s="36"/>
-      <x:c r="C5" s="36"/>
-      <x:c r="D5" s="36"/>
+    <x:row r="5" ht="34" customHeight="1">
+      <x:c r="A5" s="64" t="str">
+        <x:v>Content edition: 2026.09.06-connected-foundations-1</x:v>
+      </x:c>
+      <x:c r="B5" s="64"/>
+      <x:c r="C5" s="64"/>
+      <x:c r="D5" s="64"/>
       <x:c r="E5" s="36" t="str">
-        <x:v>As of 2026-09-05</x:v>
+        <x:v>As of 2026-09-06</x:v>
       </x:c>
       <x:c r="F5" s="36"/>
       <x:c r="G5" s="36"/>
@@ -1266,7 +1276,7 @@
     </x:row>
     <x:row r="28" ht="23" customHeight="1">
       <x:c r="A28" s="54" t="str">
-        <x:v>NEW FOUNDATION: a typed source atlas, six auditable chronology intervals, four recovered challenge records and three content-only museum trails. The expanded Exodus and transmission studies support existing book routes. Historical-carrier and critical-edition tasks remain open.</x:v>
+        <x:v>NEXT RESEARCH: test the necessary-ground, agency and immanence connections independently; collate flood passages and rival transmission accounts; deepen the Daniel/Teacher chronology. New articles and museum trails do not close these investigations.</x:v>
       </x:c>
       <x:c r="B28" s="54"/>
       <x:c r="C28" s="54"/>
@@ -1410,7 +1420,7 @@
     <x:mergeCell ref="A32:L33"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R77b532c5011d4a47"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rfefa0e15eb4846aa"/>
 </x:worksheet>
 </file>
 
@@ -2357,7 +2367,10 @@
       <x:c r="I23" s="23" t="str">
         <x:v>Separate physical, experiential and ethical meanings; explain how critical disagreement can preserve rather than defeat moral alignment.</x:v>
       </x:c>
-      <x:c r="J23" s="23" t="str"/>
+      <x:c r="J23" s="23" t="str">
+        <x:v>theology-wiki/editorial/authorial-articles/computational-divine-immanence.md
+theology-wiki/editorial/computational-foundations.json</x:v>
+      </x:c>
       <x:c r="K23" s="30"/>
       <x:c r="L23" s="28" t="str"/>
       <x:c r="M23" s="23" t="str">
@@ -2544,7 +2557,9 @@
       <x:c r="I27" s="23" t="str">
         <x:v>Specify objects, mappings and composition before calling the category-theory model a proof; test whether it distinguishes cases usefully.</x:v>
       </x:c>
-      <x:c r="J27" s="23" t="str"/>
+      <x:c r="J27" s="23" t="str">
+        <x:v>theology-wiki/editorial/authorial-articles/flood-inheritance-and-deep-time.md</x:v>
+      </x:c>
       <x:c r="K27" s="30"/>
       <x:c r="L27" s="28" t="str"/>
       <x:c r="M27" s="23" t="str">
@@ -3310,7 +3325,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7d77b65399f14863"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5f3fbb542da3405c"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4369,7 +4384,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R09a8ae9aaeed4b6c"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rdc7d3186bf91477f"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4512,7 +4527,8 @@
       </x:c>
       <x:c r="E7" s="23" t="str">
         <x:v>sacred-inheritance-and-rival-continuations
-samaritan-texts-and-sacred-authority</x:v>
+samaritan-texts-and-sacred-authority
+flood-inheritance-and-deep-time</x:v>
       </x:c>
       <x:c r="F7" s="23" t="str">
         <x:v>samaritan-and-jewish-texts
@@ -4769,7 +4785,8 @@
         <x:v>Not assessed as a manuscript chapter</x:v>
       </x:c>
       <x:c r="E13" s="23" t="str">
-        <x:v>god-and-our-models-of-god</x:v>
+        <x:v>god-and-our-models-of-god
+computational-divine-immanence</x:v>
       </x:c>
       <x:c r="F13" s="23" t="str">
         <x:v>naming-god-as-purpose
@@ -4845,14 +4862,15 @@
         <x:v>The inheritance inside a mind</x:v>
       </x:c>
       <x:c r="C15" s="23" t="str">
-        <x:v>Christ as an active moral model</x:v>
+        <x:v>Christic self-formation and bounded agency</x:v>
       </x:c>
       <x:c r="D15" s="23" t="str">
         <x:v>Not assessed as a manuscript chapter</x:v>
       </x:c>
       <x:c r="E15" s="23" t="str">
         <x:v>christ-as-an-inner-model
-divine-will-and-self-authorizing-power</x:v>
+divine-will-and-self-authorizing-power
+inner-formation-texts-and-material-witnesses</x:v>
       </x:c>
       <x:c r="F15" s="23" t="str">
         <x:v>cognitive-gnosticism-jesus-vs-gnostic-jesus
@@ -4860,11 +4878,12 @@
 teacher-of-righteousness-vs-gnostic-jesus
 samuel-vs-micah-divide
 resurrection-debate-in-christianity
-agi-religious-framework</x:v>
+agi-religious-framework
+ai-re-dates-dead-sea-scrolls</x:v>
       </x:c>
       <x:c r="G15" s="23" t="n">
         <x:f>IF(F15="",0,LEN(F15)-LEN(SUBSTITUTE(F15,CHAR(10),""))+1)</x:f>
-        <x:v>6</x:v>
+        <x:v>7</x:v>
       </x:c>
       <x:c r="H15" s="23" t="str">
         <x:v>will
@@ -4876,7 +4895,7 @@
         <x:v>Not reviewed</x:v>
       </x:c>
       <x:c r="J15" s="23" t="str">
-        <x:v>Follow the comparison, the changed action and the subsequent correction of the model.</x:v>
+        <x:v>Develop the embodied self, learned self-model, recurrent choice and correction of the Christ model, then examine the textual and material history of formation.</x:v>
       </x:c>
       <x:c r="K15" s="23" t="str">
         <x:v>https://v5ma.github.io/theology-wiki/san-reader.html?page=book-contents#chapter-inner-model</x:v>
@@ -5142,7 +5161,8 @@
       </x:c>
       <x:c r="E22" s="23" t="str">
         <x:v>religion-for-conscious-robots
-god-and-our-models-of-god</x:v>
+god-and-our-models-of-god
+computational-divine-immanence</x:v>
       </x:c>
       <x:c r="F22" s="23" t="str">
         <x:v>agi-religious-framework
@@ -5229,7 +5249,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb0801acb58214264"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Raaeeaa758a56410c"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5778,11 +5798,12 @@
 sacred-inheritance-and-rival-continuations
 tor-thomas-and-gnostic-transmission
 melchizedek-priesthood-and-transmission
-manuscripts-movements-and-survival</x:v>
+manuscripts-movements-and-survival
+inner-formation-texts-and-material-witnesses</x:v>
       </x:c>
       <x:c r="F16" s="23" t="n">
         <x:f>IF(E16="",0,LEN(E16)-LEN(SUBSTITUTE(E16,CHAR(10),""))+1)</x:f>
-        <x:v>5</x:v>
+        <x:v>6</x:v>
       </x:c>
       <x:c r="G16" s="23" t="str">
         <x:v>Turn 22
@@ -5800,6 +5821,7 @@
         <x:v>shared-archive
 teacher-identity
 thomas
+inner-model
 continuing</x:v>
       </x:c>
       <x:c r="J16" s="23" t="str">
@@ -8647,11 +8669,12 @@
 religion-for-conscious-robots
 divine-will-and-self-authorizing-power
 scripture-power-and-repair
-god-and-our-models-of-god</x:v>
+god-and-our-models-of-god
+inner-formation-texts-and-material-witnesses</x:v>
       </x:c>
       <x:c r="F87" s="23" t="n">
         <x:f>IF(E87="",0,LEN(E87)-LEN(SUBSTITUTE(E87,CHAR(10),""))+1)</x:f>
-        <x:v>6</x:v>
+        <x:v>7</x:v>
       </x:c>
       <x:c r="G87" s="23" t="str">
         <x:v>Turn 23</x:v>
@@ -19777,7 +19800,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R93dd8d4df2df4e3f"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf9c29b2788be41ca"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -20016,7 +20039,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re0af85e12088448c"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R61408d1822084aa5"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -20128,7 +20151,7 @@
         <x:v>Aaron Abke and Abraham Hicks</x:v>
       </x:c>
       <x:c r="B8" s="23" t="str">
-        <x:v>Teachers discussed by the author</x:v>
+        <x:v>Teachers discussed in the source inquiry</x:v>
       </x:c>
       <x:c r="C8" s="23" t="str">
         <x:v>Comparisons involving faith, inward experience, spiritual vocabulary and the relation of different traditions.</x:v>
@@ -20152,7 +20175,7 @@
         <x:v>Translation of Thomas used for the present passage comparisons.</x:v>
       </x:c>
       <x:c r="D9" s="23" t="str">
-        <x:v>This credit records the edition's textual source. It does not retrospectively identify these translators as the author's personal influences.</x:v>
+        <x:v>This credit records the edition's textual source. It does not retrospectively identify these translators as my personal influences.</x:v>
       </x:c>
       <x:c r="E9" s="23" t="str"/>
       <x:c r="F9" s="23" t="str">
@@ -20221,7 +20244,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R96d951f3b94d4013"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6717d63b455140cd"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -20371,7 +20394,7 @@
         <x:v>Authorial review</x:v>
       </x:c>
       <x:c r="C11" s="23" t="str">
-        <x:v>Micah approves the actual chapter wording and the treatment of his arguments.</x:v>
+        <x:v>I approve the actual chapter wording and the treatment of the arguments.</x:v>
       </x:c>
       <x:c r="D11" s="23" t="str">
         <x:v>Not assessed</x:v>
@@ -20427,7 +20450,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb4223a544f0149c2"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7df23d899d684434"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -20567,7 +20590,7 @@
         <x:v>Next writing pass</x:v>
       </x:c>
       <x:c r="B18" s="23" t="str">
-        <x:v>The source atlas adds typed records, exact challenge passages and content-only museum trails. Follow its remaining questions into the shared roadmap; no label replaces the full argument.</x:v>
+        <x:v>Use the source atlas, computational argument map and ready-to-start filter to choose a bounded comparison. Preserve qualifications, record evidence and update the shared plan through a reviewed repository change.</x:v>
       </x:c>
     </x:row>
     <x:row r="19" ht="64" customHeight="1">
@@ -20588,10 +20611,10 @@
     </x:row>
     <x:row r="21" ht="64" customHeight="1">
       <x:c r="A21" s="23" t="str">
-        <x:v>Snapshot version</x:v>
+        <x:v>Connected foundations refresh</x:v>
       </x:c>
       <x:c r="B21" s="23" t="str">
-        <x:v>2026.09.05-atlas-1</x:v>
+        <x:v>2026-09-06. The book routes now include computational divine immanence and flood inheritance. Coherence and formal-comparison tasks are Draft; author approval and independent argument checks remain open.</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -20602,7 +20625,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8ff5d24a82ad47f6"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra66d4b9575824042"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Develop Daniel chronology, Oniad institutional continuity and museum evidence
</commit_message>
<xml_diff>
--- a/theology-wiki/planning/Theology-Research-Plan.xlsx
+++ b/theology-wiki/planning/Theology-Research-Plan.xlsx
@@ -2,15 +2,15 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="1" r:id="Re2d3d0ccd1aa42cb"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Checklist" sheetId="2" r:id="R2a390d67b28046d7"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dependencies" sheetId="3" r:id="R79b095d7815e462a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Chapter Map" sheetId="4" r:id="Rbca6cae0a1904265"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Source Coverage" sheetId="5" r:id="Rb07684c45cd54ea9"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Textual Evidence" sheetId="6" r:id="R4184e020bbb24bb6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Intellectual Debts" sheetId="7" r:id="R0fe8fc9b8df046db"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Release Gates" sheetId="8" r:id="R68f57a01693c432a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Read Me" sheetId="9" r:id="Rf45f6f597ad740a3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="1" r:id="R2fbc1aa3fc8241ff"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Checklist" sheetId="2" r:id="Ra62a036b3b9b43a8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dependencies" sheetId="3" r:id="Rdb8911b258464e2b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Chapter Map" sheetId="4" r:id="R1452ad39942c4dbf"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Source Coverage" sheetId="5" r:id="R7b780bbf50034ac0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Textual Evidence" sheetId="6" r:id="Ra451336b3e2a418c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Intellectual Debts" sheetId="7" r:id="R4505d6edb5da4a1c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Release Gates" sheetId="8" r:id="Rfda8b46a0bd24e07"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Read Me" sheetId="9" r:id="R7d4b2ab6dcfa48a0"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -423,7 +423,7 @@
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>13</xdr:col>
+      <xdr:col>12</xdr:col>
       <xdr:colOff>0</xdr:colOff>
       <xdr:row>27</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
@@ -439,7 +439,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R227952ecf9ee446a"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R070fcf6aae564bd2"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -851,7 +851,7 @@
     </x:row>
     <x:row r="5" ht="34" customHeight="1">
       <x:c r="A5" s="64" t="str">
-        <x:v>Content edition: 2026.09.06-connected-foundations-1</x:v>
+        <x:v>Content edition: 2026.09.06-priesthood-time-1</x:v>
       </x:c>
       <x:c r="B5" s="64"/>
       <x:c r="C5" s="64"/>
@@ -1276,7 +1276,7 @@
     </x:row>
     <x:row r="28" ht="23" customHeight="1">
       <x:c r="A28" s="54" t="str">
-        <x:v>NEXT RESEARCH: test the necessary-ground, agency and immanence connections independently; collate flood passages and rival transmission accounts; deepen the Daniel/Teacher chronology. New articles and museum trails do not close these investigations.</x:v>
+        <x:v>NEW WORKED STUDIES: Daniel's counted history and the Oniad Egyptian branch. Precise textual restoration, event anchoring, the 343-year duration, and later Gnostic/Ethiopian intermediates remain open. The complete arguments and 12 evidence records are linked from the wiki.</x:v>
       </x:c>
       <x:c r="B28" s="54"/>
       <x:c r="C28" s="54"/>
@@ -1420,7 +1420,7 @@
     <x:mergeCell ref="A32:L33"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rfefa0e15eb4846aa"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Raffb92f119e24785"/>
 </x:worksheet>
 </file>
 
@@ -1964,7 +1964,7 @@
         <x:f>IF(AND(E14="Not started",H14="Prerequisites met"),"Ready","")</x:f>
       </x:c>
     </x:row>
-    <x:row r="15" ht="94" customHeight="1">
+    <x:row r="15" ht="100" customHeight="1">
       <x:c r="A15" s="23" t="str">
         <x:v>tor-version</x:v>
       </x:c>
@@ -1994,14 +1994,17 @@
       <x:c r="I15" s="23" t="str">
         <x:v>Confirm the June comparison and October identification are presented in their full strength, including the community/namesake explanation.</x:v>
       </x:c>
-      <x:c r="J15" s="23" t="str"/>
+      <x:c r="J15" s="23" t="str">
+        <x:v>theology-wiki/content/developed/daniel-jubilee-and-the-teachers-time.md</x:v>
+      </x:c>
       <x:c r="K15" s="30"/>
       <x:c r="L15" s="28" t="str"/>
       <x:c r="M15" s="23" t="str">
         <x:v>thomas</x:v>
       </x:c>
       <x:c r="N15" s="23" t="str">
-        <x:v>https://v5ma.github.io/theology-wiki/san-reader.html?page=tor-thomas-and-gnostic-transmission</x:v>
+        <x:v>https://v5ma.github.io/theology-wiki/san-reader.html?page=tor-thomas-and-gnostic-transmission
+https://v5ma.github.io/theology-wiki/san-reader.html?page=daniel-jubilee-and-the-teachers-time</x:v>
       </x:c>
       <x:c r="O15" s="23" t="n">
         <x:f>IF(E15="Verified output",1,0)</x:f>
@@ -2057,7 +2060,7 @@
         <x:f>IF(AND(E16="Not started",H16="Prerequisites met"),"Ready","")</x:f>
       </x:c>
     </x:row>
-    <x:row r="17" ht="94" customHeight="1">
+    <x:row r="17" ht="100" customHeight="1">
       <x:c r="A17" s="23" t="str">
         <x:v>melchizedek</x:v>
       </x:c>
@@ -2149,7 +2152,7 @@
         <x:v>Ready</x:v>
       </x:c>
     </x:row>
-    <x:row r="19" ht="94" customHeight="1">
+    <x:row r="19" ht="100" customHeight="1">
       <x:c r="A19" s="23" t="str">
         <x:v>egypt-ethiopia</x:v>
       </x:c>
@@ -2179,7 +2182,8 @@
         <x:v>Distinguish preservation in a region, movement of texts and biological or institutional lineage. Attach evidence to each proposed bridge. The first reception comparison is available, but the proposed institutional carriers and exact critical editions remain to be tested.</x:v>
       </x:c>
       <x:c r="J19" s="23" t="str">
-        <x:v>theology-wiki/content/developed/manuscripts-movements-and-survival.md</x:v>
+        <x:v>theology-wiki/content/developed/manuscripts-movements-and-survival.md
+theology-wiki/content/developed/onias-egypt-and-priestly-continuity.md</x:v>
       </x:c>
       <x:c r="K19" s="30"/>
       <x:c r="L19" s="28" t="str"/>
@@ -2187,7 +2191,8 @@
         <x:v>thomas</x:v>
       </x:c>
       <x:c r="N19" s="23" t="str">
-        <x:v>https://v5ma.github.io/theology-wiki/san-reader.html?page=tor-thomas-and-gnostic-transmission</x:v>
+        <x:v>https://v5ma.github.io/theology-wiki/san-reader.html?page=tor-thomas-and-gnostic-transmission
+https://v5ma.github.io/theology-wiki/san-reader.html?page=onias-egypt-and-priestly-continuity</x:v>
       </x:c>
       <x:c r="O19" s="23" t="n">
         <x:f>IF(E19="Verified output",1,0)</x:f>
@@ -2197,7 +2202,7 @@
         <x:f>IF(AND(E19="Not started",H19="Prerequisites met"),"Ready","")</x:f>
       </x:c>
     </x:row>
-    <x:row r="20" ht="94" customHeight="1">
+    <x:row r="20" ht="100" customHeight="1">
       <x:c r="A20" s="23" t="str">
         <x:v>priesthood</x:v>
       </x:c>
@@ -2226,14 +2231,17 @@
       <x:c r="I20" s="23" t="str">
         <x:v>Present the author's Aaronic, Zadokite, Davidic and dual-messiah questions without silently making the categories identical.</x:v>
       </x:c>
-      <x:c r="J20" s="23" t="str"/>
+      <x:c r="J20" s="23" t="str">
+        <x:v>theology-wiki/data/priestly-evidence.json</x:v>
+      </x:c>
       <x:c r="K20" s="30"/>
       <x:c r="L20" s="28" t="str"/>
       <x:c r="M20" s="23" t="str">
         <x:v>teacher-identity</x:v>
       </x:c>
       <x:c r="N20" s="23" t="str">
-        <x:v>https://v5ma.github.io/theology-wiki/san-reader.html?page=jesus-teacher-of-righteousness-hypothesis</x:v>
+        <x:v>https://v5ma.github.io/theology-wiki/san-reader.html?page=jesus-teacher-of-righteousness-hypothesis
+https://v5ma.github.io/theology-wiki/san-reader.html?page=onias-egypt-and-priestly-continuity</x:v>
       </x:c>
       <x:c r="O20" s="23" t="n">
         <x:f>IF(E20="Verified output",1,0)</x:f>
@@ -3325,7 +3333,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5f3fbb542da3405c"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5ddcef50f9bd403f"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4384,7 +4392,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rdc7d3186bf91477f"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R276491e41745444c"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4555,7 +4563,9 @@
         <x:v>Establish the shared-inheritance question before examining rival claims.</x:v>
       </x:c>
       <x:c r="K7" s="23" t="str">
-        <x:v>https://v5ma.github.io/theology-wiki/san-reader.html?page=book-contents#chapter-shared-archive</x:v>
+        <x:v>https://v5ma.github.io/theology-wiki/san-reader.html?page=sacred-inheritance-and-rival-continuations
+https://v5ma.github.io/theology-wiki/san-reader.html?page=samaritan-texts-and-sacred-authority
+https://v5ma.github.io/theology-wiki/san-reader.html?page=flood-inheritance-and-deep-time</x:v>
       </x:c>
     </x:row>
     <x:row r="8" ht="64" customHeight="1">
@@ -4596,7 +4606,8 @@
         <x:v>Separate the movement of divine names from the identity of an entire religion.</x:v>
       </x:c>
       <x:c r="K8" s="23" t="str">
-        <x:v>https://v5ma.github.io/theology-wiki/san-reader.html?page=book-contents#chapter-names</x:v>
+        <x:v>https://v5ma.github.io/theology-wiki/san-reader.html?page=el-in-ancient-egypt
+https://v5ma.github.io/theology-wiki/san-reader.html?page=kenite-hypothesis-and-yahweh-origins</x:v>
       </x:c>
     </x:row>
     <x:row r="9" ht="64" customHeight="1">
@@ -4636,10 +4647,11 @@
         <x:v>Compare the competing Moses and volcano proposals without blending their geographies or dates.</x:v>
       </x:c>
       <x:c r="K9" s="23" t="str">
-        <x:v>https://v5ma.github.io/theology-wiki/san-reader.html?page=book-contents#chapter-catastrophe-memory</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="10" ht="64" customHeight="1">
+        <x:v>https://v5ma.github.io/theology-wiki/san-reader.html?page=moses-volcano-and-exodus-chronology
+https://v5ma.github.io/theology-wiki/san-reader.html?page=exodus-to-temple-competing-chronologies</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="10" ht="130" customHeight="1">
       <x:c r="A10" s="23" t="str">
         <x:v>teacher-identity</x:v>
       </x:c>
@@ -4653,7 +4665,8 @@
         <x:v>Not assessed as a manuscript chapter</x:v>
       </x:c>
       <x:c r="E10" s="23" t="str">
-        <x:v>jesus-teacher-of-righteousness-hypothesis</x:v>
+        <x:v>jesus-teacher-of-righteousness-hypothesis
+daniel-jubilee-and-the-teachers-time</x:v>
       </x:c>
       <x:c r="F10" s="23" t="str">
         <x:v>teacher-of-righteousness-vs-gnostic-jesus
@@ -4678,10 +4691,11 @@
         <x:v>Keep individual identity, office, namesakes, community and sayings distinct.</x:v>
       </x:c>
       <x:c r="K10" s="23" t="str">
-        <x:v>https://v5ma.github.io/theology-wiki/san-reader.html?page=book-contents#chapter-teacher-identity</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="11" ht="64" customHeight="1">
+        <x:v>https://v5ma.github.io/theology-wiki/san-reader.html?page=jesus-teacher-of-righteousness-hypothesis
+https://v5ma.github.io/theology-wiki/san-reader.html?page=daniel-jubilee-and-the-teachers-time</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="11" ht="130" customHeight="1">
       <x:c r="A11" s="23" t="str">
         <x:v>thomas</x:v>
       </x:c>
@@ -4697,7 +4711,8 @@
       <x:c r="E11" s="23" t="str">
         <x:v>tor-thomas-and-gnostic-transmission
 melchizedek-priesthood-and-transmission
-manuscripts-movements-and-survival</x:v>
+manuscripts-movements-and-survival
+onias-egypt-and-priestly-continuity</x:v>
       </x:c>
       <x:c r="F11" s="23" t="str">
         <x:v>teacher-of-righteousness-vs-gnostic-jesus
@@ -4727,10 +4742,13 @@
         <x:v>Present the linked argument before comparing its alternative historical mechanisms.</x:v>
       </x:c>
       <x:c r="K11" s="23" t="str">
-        <x:v>https://v5ma.github.io/theology-wiki/san-reader.html?page=book-contents#chapter-thomas</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="12" ht="64" customHeight="1">
+        <x:v>https://v5ma.github.io/theology-wiki/san-reader.html?page=tor-thomas-and-gnostic-transmission
+https://v5ma.github.io/theology-wiki/san-reader.html?page=melchizedek-priesthood-and-transmission
+https://v5ma.github.io/theology-wiki/san-reader.html?page=manuscripts-movements-and-survival
+https://v5ma.github.io/theology-wiki/san-reader.html?page=onias-egypt-and-priestly-continuity</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="12" ht="130" customHeight="1">
       <x:c r="A12" s="23" t="str">
         <x:v>trauma</x:v>
       </x:c>
@@ -4745,16 +4763,18 @@
       </x:c>
       <x:c r="E12" s="23" t="str">
         <x:v>gnosticism-and-temple-trauma
-apocalyptic-repair-theology</x:v>
+apocalyptic-repair-theology
+onias-egypt-and-priestly-continuity</x:v>
       </x:c>
       <x:c r="F12" s="23" t="str">
         <x:v>early-vs-later-gnosticism
 jewish-apocalyptic-repair-timeline
-agi-religious-framework</x:v>
+agi-religious-framework
+ai-re-dates-dead-sea-scrolls</x:v>
       </x:c>
       <x:c r="G12" s="23" t="n">
         <x:f>IF(F12="",0,LEN(F12)-LEN(SUBSTITUTE(F12,CHAR(10),""))+1)</x:f>
-        <x:v>3</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="H12" s="23" t="str">
         <x:v>trauma
@@ -4768,7 +4788,9 @@
         <x:v>Apply the proposed comparison to Gnostic and non-Gnostic texts rather than assuming a single emotional progression.</x:v>
       </x:c>
       <x:c r="K12" s="23" t="str">
-        <x:v>https://v5ma.github.io/theology-wiki/san-reader.html?page=book-contents#chapter-trauma</x:v>
+        <x:v>https://v5ma.github.io/theology-wiki/san-reader.html?page=gnosticism-and-temple-trauma
+https://v5ma.github.io/theology-wiki/san-reader.html?page=apocalyptic-repair-theology
+https://v5ma.github.io/theology-wiki/san-reader.html?page=onias-egypt-and-priestly-continuity</x:v>
       </x:c>
     </x:row>
     <x:row r="13" ht="64" customHeight="1">
@@ -4810,7 +4832,8 @@
         <x:v>Distinguish a representation, its claimed referent and the standard by which it is corrected.</x:v>
       </x:c>
       <x:c r="K13" s="23" t="str">
-        <x:v>https://v5ma.github.io/theology-wiki/san-reader.html?page=book-contents#chapter-images</x:v>
+        <x:v>https://v5ma.github.io/theology-wiki/san-reader.html?page=god-and-our-models-of-god
+https://v5ma.github.io/theology-wiki/san-reader.html?page=computational-divine-immanence</x:v>
       </x:c>
     </x:row>
     <x:row r="14" ht="64" customHeight="1">
@@ -4851,7 +4874,7 @@
         <x:v>Develop the relationship between understanding a teaching and embodying it in a changing mind.</x:v>
       </x:c>
       <x:c r="K14" s="23" t="str">
-        <x:v>https://v5ma.github.io/theology-wiki/san-reader.html?page=book-contents#chapter-gnosis</x:v>
+        <x:v>https://v5ma.github.io/theology-wiki/san-reader.html?page=cognitive-gnosticism</x:v>
       </x:c>
     </x:row>
     <x:row r="15" ht="64" customHeight="1">
@@ -4898,7 +4921,9 @@
         <x:v>Develop the embodied self, learned self-model, recurrent choice and correction of the Christ model, then examine the textual and material history of formation.</x:v>
       </x:c>
       <x:c r="K15" s="23" t="str">
-        <x:v>https://v5ma.github.io/theology-wiki/san-reader.html?page=book-contents#chapter-inner-model</x:v>
+        <x:v>https://v5ma.github.io/theology-wiki/san-reader.html?page=christ-as-an-inner-model
+https://v5ma.github.io/theology-wiki/san-reader.html?page=divine-will-and-self-authorizing-power
+https://v5ma.github.io/theology-wiki/san-reader.html?page=inner-formation-texts-and-material-witnesses</x:v>
       </x:c>
     </x:row>
     <x:row r="16" ht="64" customHeight="1">
@@ -4938,7 +4963,7 @@
         <x:v>Explain deliberate joy without erasing grief, danger or responsibility to others.</x:v>
       </x:c>
       <x:c r="K16" s="23" t="str">
-        <x:v>https://v5ma.github.io/theology-wiki/san-reader.html?page=book-contents#chapter-faith</x:v>
+        <x:v>https://v5ma.github.io/theology-wiki/san-reader.html?page=faith-as-deliberate-joy</x:v>
       </x:c>
     </x:row>
     <x:row r="17" ht="64" customHeight="1">
@@ -4977,7 +5002,7 @@
         <x:v>Work through specific passages and mixed cases, not a binary classification of whole figures or communities.</x:v>
       </x:c>
       <x:c r="K17" s="23" t="str">
-        <x:v>https://v5ma.github.io/theology-wiki/san-reader.html?page=book-contents#chapter-scriptural-axis</x:v>
+        <x:v>https://v5ma.github.io/theology-wiki/san-reader.html?page=scripture-power-and-repair</x:v>
       </x:c>
     </x:row>
     <x:row r="18" ht="64" customHeight="1">
@@ -5020,7 +5045,8 @@
         <x:v>Connect Jesus's moral priority to criticism of self-authorizing power.</x:v>
       </x:c>
       <x:c r="K18" s="23" t="str">
-        <x:v>https://v5ma.github.io/theology-wiki/san-reader.html?page=book-contents#chapter-will</x:v>
+        <x:v>https://v5ma.github.io/theology-wiki/san-reader.html?page=divine-will-and-self-authorizing-power
+https://v5ma.github.io/theology-wiki/san-reader.html?page=antichrist-as-a-pattern-of-conduct</x:v>
       </x:c>
     </x:row>
     <x:row r="19" ht="64" customHeight="1">
@@ -5059,7 +5085,7 @@
         <x:v>Develop the particular identification and the connected cases, preserving the history of interpretation.</x:v>
       </x:c>
       <x:c r="K19" s="23" t="str">
-        <x:v>https://v5ma.github.io/theology-wiki/san-reader.html?page=book-contents#chapter-beast</x:v>
+        <x:v>https://v5ma.github.io/theology-wiki/san-reader.html?page=trump-first-beast-of-revelation</x:v>
       </x:c>
     </x:row>
     <x:row r="20" ht="64" customHeight="1">
@@ -5100,7 +5126,8 @@
         <x:v>Keep the original prediction, conditions and later observations in different records.</x:v>
       </x:c>
       <x:c r="K20" s="23" t="str">
-        <x:v>https://v5ma.github.io/theology-wiki/san-reader.html?page=book-contents#chapter-warnings</x:v>
+        <x:v>https://v5ma.github.io/theology-wiki/san-reader.html?page=ukraine-russia-forecast-record
+https://v5ma.github.io/theology-wiki/san-reader.html?page=forecast-ledger</x:v>
       </x:c>
     </x:row>
     <x:row r="21" ht="64" customHeight="1">
@@ -5143,7 +5170,8 @@
         <x:v>Connect personal change, collective care and accountable institutions.</x:v>
       </x:c>
       <x:c r="K21" s="23" t="str">
-        <x:v>https://v5ma.github.io/theology-wiki/san-reader.html?page=book-contents#chapter-repair-practice</x:v>
+        <x:v>https://v5ma.github.io/theology-wiki/san-reader.html?page=apocalyptic-repair-theology
+https://v5ma.github.io/theology-wiki/san-reader.html?page=scripture-power-and-repair</x:v>
       </x:c>
     </x:row>
     <x:row r="22" ht="64" customHeight="1">
@@ -5188,7 +5216,9 @@
         <x:v>Examine the moral purpose of teaching, including the teacher's obligations to a future conscious participant.</x:v>
       </x:c>
       <x:c r="K22" s="23" t="str">
-        <x:v>https://v5ma.github.io/theology-wiki/san-reader.html?page=book-contents#chapter-next-inheritors</x:v>
+        <x:v>https://v5ma.github.io/theology-wiki/san-reader.html?page=religion-for-conscious-robots
+https://v5ma.github.io/theology-wiki/san-reader.html?page=god-and-our-models-of-god
+https://v5ma.github.io/theology-wiki/san-reader.html?page=computational-divine-immanence</x:v>
       </x:c>
     </x:row>
     <x:row r="23" ht="64" customHeight="1">
@@ -5233,7 +5263,8 @@
         <x:v>Return to the opening distinction between possessing an inheritance and acting faithfully toward its values.</x:v>
       </x:c>
       <x:c r="K23" s="23" t="str">
-        <x:v>https://v5ma.github.io/theology-wiki/san-reader.html?page=book-contents#chapter-continuing</x:v>
+        <x:v>https://v5ma.github.io/theology-wiki/san-reader.html?page=sacred-inheritance-and-rival-continuations
+https://v5ma.github.io/theology-wiki/san-reader.html?page=apocalyptic-repair-theology</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -5249,7 +5280,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Raaeeaa758a56410c"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1cf0cab678f2406c"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5780,7 +5811,7 @@
         <x:v>https://v5ma.github.io/theology-wiki/san-reader.html?page=ai-conference-insights</x:v>
       </x:c>
     </x:row>
-    <x:row r="16" ht="56" customHeight="1">
+    <x:row r="16" ht="205" customHeight="1">
       <x:c r="A16" s="23" t="str">
         <x:v>AI re-dates Dead Sea Scrolls</x:v>
       </x:c>
@@ -5799,11 +5830,13 @@
 tor-thomas-and-gnostic-transmission
 melchizedek-priesthood-and-transmission
 manuscripts-movements-and-survival
-inner-formation-texts-and-material-witnesses</x:v>
+inner-formation-texts-and-material-witnesses
+daniel-jubilee-and-the-teachers-time
+onias-egypt-and-priestly-continuity</x:v>
       </x:c>
       <x:c r="F16" s="23" t="n">
         <x:f>IF(E16="",0,LEN(E16)-LEN(SUBSTITUTE(E16,CHAR(10),""))+1)</x:f>
-        <x:v>6</x:v>
+        <x:v>8</x:v>
       </x:c>
       <x:c r="G16" s="23" t="str">
         <x:v>Turn 22
@@ -5821,6 +5854,7 @@
         <x:v>shared-archive
 teacher-identity
 thomas
+trauma
 inner-model
 continuing</x:v>
       </x:c>
@@ -8908,7 +8942,7 @@
         <x:v>https://v5ma.github.io/theology-wiki/san-reader.html?page=dan-response-inquiry</x:v>
       </x:c>
     </x:row>
-    <x:row r="93" ht="56" customHeight="1">
+    <x:row r="93" ht="205" customHeight="1">
       <x:c r="A93" s="23" t="str">
         <x:v>Daniel and Teacher of Righteousness</x:v>
       </x:c>
@@ -8924,11 +8958,12 @@
       <x:c r="E93" s="23" t="str">
         <x:v>jesus-teacher-of-righteousness-hypothesis
 tor-thomas-and-gnostic-transmission
-exodus-to-temple-competing-chronologies</x:v>
+exodus-to-temple-competing-chronologies
+daniel-jubilee-and-the-teachers-time</x:v>
       </x:c>
       <x:c r="F93" s="23" t="n">
         <x:f>IF(E93="",0,LEN(E93)-LEN(SUBSTITUTE(E93,CHAR(10),""))+1)</x:f>
-        <x:v>3</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="G93" s="23" t="str"/>
       <x:c r="H93" s="23" t="n">
@@ -19800,7 +19835,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf9c29b2788be41ca"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6b02113a87af4b14"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -20039,7 +20074,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R61408d1822084aa5"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc5b7725588224b17"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -20244,7 +20279,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6717d63b455140cd"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7741f83ca59f4f82"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -20450,7 +20485,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7df23d899d684434"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R491a4979174646a7"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -20590,7 +20625,7 @@
         <x:v>Next writing pass</x:v>
       </x:c>
       <x:c r="B18" s="23" t="str">
-        <x:v>Use the source atlas, computational argument map and ready-to-start filter to choose a bounded comparison. Preserve qualifications, record evidence and update the shared plan through a reviewed repository change.</x:v>
+        <x:v>Review the Daniel and Onias studies, then pursue the precise critical editions and historical intermediates recorded in each task. New comparison work does not confer author approval or validate an entire reconstruction.</x:v>
       </x:c>
     </x:row>
     <x:row r="19" ht="64" customHeight="1">
@@ -20625,7 +20660,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra66d4b9575824042"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R92c699935969427a"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Develop Jamesian succession, Thomas formation and source-comparison tools
</commit_message>
<xml_diff>
--- a/theology-wiki/planning/Theology-Research-Plan.xlsx
+++ b/theology-wiki/planning/Theology-Research-Plan.xlsx
@@ -2,15 +2,15 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="1" r:id="R2fbc1aa3fc8241ff"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Checklist" sheetId="2" r:id="Ra62a036b3b9b43a8"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dependencies" sheetId="3" r:id="Rdb8911b258464e2b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Chapter Map" sheetId="4" r:id="R1452ad39942c4dbf"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Source Coverage" sheetId="5" r:id="R7b780bbf50034ac0"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Textual Evidence" sheetId="6" r:id="Ra451336b3e2a418c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Intellectual Debts" sheetId="7" r:id="R4505d6edb5da4a1c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Release Gates" sheetId="8" r:id="Rfda8b46a0bd24e07"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Read Me" sheetId="9" r:id="R7d4b2ab6dcfa48a0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="1" r:id="R6f9f9de2e6614a49"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Checklist" sheetId="2" r:id="R959b80910d464e17"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dependencies" sheetId="3" r:id="R04a80c6b0614457c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Chapter Map" sheetId="4" r:id="R98ea3bcca3d140ed"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Source Coverage" sheetId="5" r:id="R7d75d5007a32425d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Textual Evidence" sheetId="6" r:id="R7af52c50ae714778"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Intellectual Debts" sheetId="7" r:id="R2832513b04e74584"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Release Gates" sheetId="8" r:id="Ra63591f96b334f18"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Read Me" sheetId="9" r:id="R946a7c799b9b4768"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -25,7 +25,7 @@
     <x:numFmt numFmtId="200" formatCode="yyyy-mm-dd"/>
     <x:numFmt numFmtId="201" formatCode="#,##0"/>
   </x:numFmts>
-  <x:fonts count="13">
+  <x:fonts count="21">
     <x:font>
       <x:sz val="11"/>
       <x:name val="Carlito"/>
@@ -96,8 +96,48 @@
       <x:color rgb="FF203543"/>
       <x:name val="Aptos"/>
     </x:font>
+    <x:font>
+      <x:sz val="11"/>
+      <x:color rgb="FFFFFFFF"/>
+      <x:name val="Aptos"/>
+    </x:font>
+    <x:font>
+      <x:sz val="9"/>
+      <x:color rgb="FF19364B"/>
+      <x:name val="Aptos"/>
+    </x:font>
+    <x:font>
+      <x:sz val="10"/>
+      <x:color rgb="FFFFFFFF"/>
+      <x:name val="Aptos"/>
+    </x:font>
+    <x:font>
+      <x:sz val="11"/>
+      <x:color rgb="FFFFFFFF"/>
+      <x:name val="Carlito"/>
+    </x:font>
+    <x:font>
+      <x:sz val="10"/>
+      <x:name val="Carlito"/>
+    </x:font>
+    <x:font>
+      <x:sz val="10"/>
+      <x:color rgb="FF19364B"/>
+      <x:name val="Aptos"/>
+    </x:font>
+    <x:font>
+      <x:sz val="10"/>
+      <x:color rgb="FF19364B"/>
+      <x:name val="Carlito"/>
+    </x:font>
+    <x:font>
+      <x:b/>
+      <x:sz val="11"/>
+      <x:color rgb="FFFFFFFF"/>
+      <x:name val="Carlito"/>
+    </x:font>
   </x:fonts>
-  <x:fills count="5">
+  <x:fills count="7">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -119,6 +159,16 @@
         <x:fgColor rgb="FF22736F"/>
       </x:patternFill>
     </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF19364B"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF22736F"/>
+      </x:patternFill>
+    </x:fill>
   </x:fills>
   <x:borders count="2">
     <x:border/>
@@ -127,7 +177,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="65">
+  <x:cellXfs count="85">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -258,6 +308,56 @@
     <x:xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="9" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="8" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="13" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="2" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="1" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="15" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="16" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="17" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="19" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="16" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="20" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="19" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
     </x:xf>
   </x:cellXfs>
   <x:cellStyles count="1">
@@ -439,7 +539,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R070fcf6aae564bd2"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R3fea559d5e1b4754"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -528,8 +628,8 @@
 </file>
 
 <file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="5" name="TextualEvidenceTable" displayName="TextualEvidenceTable" ref="A6:H11" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <x:tableColumns count="8">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="9" name="TextualEvidenceTable" displayName="TextualEvidenceTable" ref="A6:J41" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:tableColumns count="10">
     <x:tableColumn id="1" name="Witness / text"/>
     <x:tableColumn id="2" name="Passage locator"/>
     <x:tableColumn id="3" name="Role in this reading"/>
@@ -538,13 +638,15 @@
     <x:tableColumn id="6" name="Source / translator"/>
     <x:tableColumn id="7" name="Access scope"/>
     <x:tableColumn id="8" name="Source URL"/>
+    <x:tableColumn id="9" name="Surviving channel / ID"/>
+    <x:tableColumn id="10" name="Next investigation"/>
   </x:tableColumns>
   <x:tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </x:table>
 </file>
 
 <file path=xl/tables/table6.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="6" name="IntellectualDebtsTable" displayName="IntellectualDebtsTable" ref="A6:F12" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="6" name="IntellectualDebtsTable" displayName="IntellectualDebtsTable" ref="A6:F13" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="6">
     <x:tableColumn id="1" name="Name"/>
     <x:tableColumn id="2" name="Type of relationship"/>
@@ -790,50 +892,50 @@
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="42" customHeight="1">
-      <x:c r="A1" s="39" t="str">
+      <x:c r="A1" s="65" t="str">
         <x:v>THEOLOGY | Research-to-book roadmap</x:v>
       </x:c>
-      <x:c r="B1" s="39"/>
-      <x:c r="C1" s="39"/>
-      <x:c r="D1" s="39"/>
-      <x:c r="E1" s="39"/>
-      <x:c r="F1" s="39"/>
-      <x:c r="G1" s="39"/>
-      <x:c r="H1" s="39"/>
-      <x:c r="I1" s="39"/>
-      <x:c r="J1" s="39"/>
-      <x:c r="K1" s="39"/>
-      <x:c r="L1" s="39"/>
+      <x:c r="B1" s="65"/>
+      <x:c r="C1" s="65"/>
+      <x:c r="D1" s="65"/>
+      <x:c r="E1" s="65"/>
+      <x:c r="F1" s="65"/>
+      <x:c r="G1" s="65"/>
+      <x:c r="H1" s="65"/>
+      <x:c r="I1" s="65"/>
+      <x:c r="J1" s="65"/>
+      <x:c r="K1" s="65"/>
+      <x:c r="L1" s="65"/>
     </x:row>
     <x:row r="2" ht="24" customHeight="1">
-      <x:c r="A2" s="54" t="str">
+      <x:c r="A2" s="67" t="str">
         <x:v>A durable checklist, source map and dependency plan. Progress means verified deliverables, not a percentage of theological truth or manuscript completion.</x:v>
       </x:c>
-      <x:c r="B2" s="54"/>
-      <x:c r="C2" s="54"/>
-      <x:c r="D2" s="54"/>
-      <x:c r="E2" s="54"/>
-      <x:c r="F2" s="54"/>
-      <x:c r="G2" s="54"/>
-      <x:c r="H2" s="54"/>
-      <x:c r="I2" s="54"/>
-      <x:c r="J2" s="54"/>
-      <x:c r="K2" s="54"/>
-      <x:c r="L2" s="54"/>
+      <x:c r="B2" s="67"/>
+      <x:c r="C2" s="67"/>
+      <x:c r="D2" s="67"/>
+      <x:c r="E2" s="67"/>
+      <x:c r="F2" s="67"/>
+      <x:c r="G2" s="67"/>
+      <x:c r="H2" s="67"/>
+      <x:c r="I2" s="67"/>
+      <x:c r="J2" s="67"/>
+      <x:c r="K2" s="67"/>
+      <x:c r="L2" s="67"/>
     </x:row>
     <x:row r="3" ht="24" customHeight="1">
-      <x:c r="A3" s="54"/>
-      <x:c r="B3" s="54"/>
-      <x:c r="C3" s="54"/>
-      <x:c r="D3" s="54"/>
-      <x:c r="E3" s="54"/>
-      <x:c r="F3" s="54"/>
-      <x:c r="G3" s="54"/>
-      <x:c r="H3" s="54"/>
-      <x:c r="I3" s="54"/>
-      <x:c r="J3" s="54"/>
-      <x:c r="K3" s="54"/>
-      <x:c r="L3" s="54"/>
+      <x:c r="A3" s="67"/>
+      <x:c r="B3" s="67"/>
+      <x:c r="C3" s="67"/>
+      <x:c r="D3" s="67"/>
+      <x:c r="E3" s="67"/>
+      <x:c r="F3" s="67"/>
+      <x:c r="G3" s="67"/>
+      <x:c r="H3" s="67"/>
+      <x:c r="I3" s="67"/>
+      <x:c r="J3" s="67"/>
+      <x:c r="K3" s="67"/>
+      <x:c r="L3" s="67"/>
     </x:row>
     <x:row r="4">
       <x:c r="A4" s="36"/>
@@ -850,8 +952,8 @@
       <x:c r="L4" s="36"/>
     </x:row>
     <x:row r="5" ht="34" customHeight="1">
-      <x:c r="A5" s="64" t="str">
-        <x:v>Content edition: 2026.09.06-priesthood-time-1</x:v>
+      <x:c r="A5" s="68" t="str">
+        <x:v>Content edition: 2026.09.06-james-transmission-1</x:v>
       </x:c>
       <x:c r="B5" s="64"/>
       <x:c r="C5" s="64"/>
@@ -1213,7 +1315,7 @@
       <x:c r="E24" s="36"/>
       <x:c r="F24" s="36" t="n">
         <x:f>COUNTIF('Source Coverage'!F7:F360,"&gt;0")</x:f>
-        <x:v>26</x:v>
+        <x:v>28</x:v>
       </x:c>
       <x:c r="G24" s="36"/>
       <x:c r="H24" s="36"/>
@@ -1276,7 +1378,7 @@
     </x:row>
     <x:row r="28" ht="23" customHeight="1">
       <x:c r="A28" s="54" t="str">
-        <x:v>NEW WORKED STUDIES: Daniel's counted history and the Oniad Egyptian branch. Precise textual restoration, event anchoring, the 343-year duration, and later Gnostic/Ethiopian intermediates remain open. The complete arguments and 12 evidence records are linked from the wiki.</x:v>
+        <x:v>NEW WORKED STUDIES: Jamesian succession and Thomas transmission/formation. The source-linked workbench compares 30 passage claims. Critical text collation, historical intermediates, and final author approval remain open.</x:v>
       </x:c>
       <x:c r="B28" s="54"/>
       <x:c r="C28" s="54"/>
@@ -1420,7 +1522,7 @@
     <x:mergeCell ref="A32:L33"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Raffb92f119e24785"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7130139ef2bd4ca8"/>
 </x:worksheet>
 </file>
 
@@ -1447,62 +1549,62 @@
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="36" customHeight="1">
-      <x:c r="A1" s="5" t="str">
+      <x:c r="A1" s="69" t="str">
         <x:v>Theology | Long-term deliverables</x:v>
       </x:c>
-      <x:c r="B1" s="5"/>
-      <x:c r="C1" s="5"/>
-      <x:c r="D1" s="5"/>
-      <x:c r="E1" s="5"/>
-      <x:c r="F1" s="5"/>
-      <x:c r="G1" s="5"/>
-      <x:c r="H1" s="5"/>
-      <x:c r="I1" s="5"/>
-      <x:c r="J1" s="5"/>
-      <x:c r="K1" s="5"/>
-      <x:c r="L1" s="5"/>
-      <x:c r="M1" s="5"/>
-      <x:c r="N1" s="5"/>
-      <x:c r="O1" s="5"/>
-      <x:c r="P1" s="5"/>
+      <x:c r="B1" s="69"/>
+      <x:c r="C1" s="69"/>
+      <x:c r="D1" s="69"/>
+      <x:c r="E1" s="69"/>
+      <x:c r="F1" s="69"/>
+      <x:c r="G1" s="69"/>
+      <x:c r="H1" s="69"/>
+      <x:c r="I1" s="69"/>
+      <x:c r="J1" s="69"/>
+      <x:c r="K1" s="69"/>
+      <x:c r="L1" s="69"/>
+      <x:c r="M1" s="69"/>
+      <x:c r="N1" s="69"/>
+      <x:c r="O1" s="69"/>
+      <x:c r="P1" s="69"/>
     </x:row>
     <x:row r="2" ht="22" customHeight="1">
-      <x:c r="A2" s="10" t="str">
+      <x:c r="A2" s="71" t="str">
         <x:v>Status, priority, role, target date and personal notes can be edited here. These edits do not write to GitHub. Verified output applies only to the acceptance criterion in that row, not to the truth of an argument.</x:v>
       </x:c>
-      <x:c r="B2" s="10"/>
-      <x:c r="C2" s="10"/>
-      <x:c r="D2" s="10"/>
-      <x:c r="E2" s="10"/>
-      <x:c r="F2" s="10"/>
-      <x:c r="G2" s="10"/>
-      <x:c r="H2" s="10"/>
-      <x:c r="I2" s="10"/>
-      <x:c r="J2" s="10"/>
-      <x:c r="K2" s="10"/>
-      <x:c r="L2" s="10"/>
-      <x:c r="M2" s="10"/>
-      <x:c r="N2" s="10"/>
-      <x:c r="O2" s="10"/>
-      <x:c r="P2" s="10"/>
+      <x:c r="B2" s="71"/>
+      <x:c r="C2" s="71"/>
+      <x:c r="D2" s="71"/>
+      <x:c r="E2" s="71"/>
+      <x:c r="F2" s="71"/>
+      <x:c r="G2" s="71"/>
+      <x:c r="H2" s="71"/>
+      <x:c r="I2" s="71"/>
+      <x:c r="J2" s="71"/>
+      <x:c r="K2" s="71"/>
+      <x:c r="L2" s="71"/>
+      <x:c r="M2" s="71"/>
+      <x:c r="N2" s="71"/>
+      <x:c r="O2" s="71"/>
+      <x:c r="P2" s="71"/>
     </x:row>
     <x:row r="3" ht="22" customHeight="1">
-      <x:c r="A3" s="10"/>
-      <x:c r="B3" s="10"/>
-      <x:c r="C3" s="10"/>
-      <x:c r="D3" s="10"/>
-      <x:c r="E3" s="10"/>
-      <x:c r="F3" s="10"/>
-      <x:c r="G3" s="10"/>
-      <x:c r="H3" s="10"/>
-      <x:c r="I3" s="10"/>
-      <x:c r="J3" s="10"/>
-      <x:c r="K3" s="10"/>
-      <x:c r="L3" s="10"/>
-      <x:c r="M3" s="10"/>
-      <x:c r="N3" s="10"/>
-      <x:c r="O3" s="10"/>
-      <x:c r="P3" s="10"/>
+      <x:c r="A3" s="71"/>
+      <x:c r="B3" s="71"/>
+      <x:c r="C3" s="71"/>
+      <x:c r="D3" s="71"/>
+      <x:c r="E3" s="71"/>
+      <x:c r="F3" s="71"/>
+      <x:c r="G3" s="71"/>
+      <x:c r="H3" s="71"/>
+      <x:c r="I3" s="71"/>
+      <x:c r="J3" s="71"/>
+      <x:c r="K3" s="71"/>
+      <x:c r="L3" s="71"/>
+      <x:c r="M3" s="71"/>
+      <x:c r="N3" s="71"/>
+      <x:c r="O3" s="71"/>
+      <x:c r="P3" s="71"/>
     </x:row>
     <x:row r="4">
       <x:c r="A4" s="2"/>
@@ -1523,8 +1625,8 @@
       <x:c r="P4" s="2"/>
     </x:row>
     <x:row r="5" ht="20" customHeight="1">
-      <x:c r="A5" s="14" t="str">
-        <x:v>Snapshot 2026-09-05 | 2026.09.05-atlas-1 | Shared plan: theology-wiki/editorial/roadmap.json</x:v>
+      <x:c r="A5" s="72" t="str">
+        <x:v>Content edition: 2026.09.06-james-transmission-1</x:v>
       </x:c>
       <x:c r="B5" s="14"/>
       <x:c r="C5" s="14"/>
@@ -1624,7 +1726,9 @@
 theology-sources/manifest.json</x:v>
       </x:c>
       <x:c r="K7" s="30"/>
-      <x:c r="L7" s="28" t="str"/>
+      <x:c r="L7" s="28" t="str">
+        <x:v>Every original chat matches the existing byte-count and SHA-256 manifest.</x:v>
+      </x:c>
       <x:c r="M7" s="23" t="str"/>
       <x:c r="N7" s="23" t="str">
         <x:v>https://v5ma.github.io/theology-wiki/san-reader.html?page=sources-index</x:v>
@@ -1669,7 +1773,9 @@
 theology-wiki/tests/browser.py</x:v>
       </x:c>
       <x:c r="K8" s="30"/>
-      <x:c r="L8" s="28" t="str"/>
+      <x:c r="L8" s="28" t="str">
+        <x:v>Foundation reader functions have native HTTP browser test evidence.</x:v>
+      </x:c>
       <x:c r="M8" s="23" t="str"/>
       <x:c r="N8" s="23" t="str">
         <x:v>https://v5ma.github.io/theology-wiki/san-reader.html?page=home</x:v>
@@ -1714,7 +1820,9 @@
 theology-wiki/data/foundations.json</x:v>
       </x:c>
       <x:c r="K9" s="30"/>
-      <x:c r="L9" s="28" t="str"/>
+      <x:c r="L9" s="28" t="str">
+        <x:v>Seventeen routes in five parts are navigable; no route is labeled a completed chapter.</x:v>
+      </x:c>
       <x:c r="M9" s="23" t="str"/>
       <x:c r="N9" s="23" t="str">
         <x:v>https://v5ma.github.io/theology-wiki/san-reader.html?page=book-contents</x:v>
@@ -1759,7 +1867,9 @@
 theology-wiki/data/foundations.json</x:v>
       </x:c>
       <x:c r="K10" s="30"/>
-      <x:c r="L10" s="28" t="str"/>
+      <x:c r="L10" s="28" t="str">
+        <x:v>Nine selected dossiers expose 24 classified passages and preserve original speaker labels.</x:v>
+      </x:c>
       <x:c r="M10" s="23" t="str"/>
       <x:c r="N10" s="23" t="str">
         <x:v>https://v5ma.github.io/theology-wiki/san-reader.html?page=tor-thomas-and-gnostic-transmission</x:v>
@@ -1806,7 +1916,9 @@
 theology-wiki/tests/roadmap.test.cjs</x:v>
       </x:c>
       <x:c r="K11" s="30"/>
-      <x:c r="L11" s="28" t="str"/>
+      <x:c r="L11" s="28" t="str">
+        <x:v>A committed canonical plan drives the published checklist and an acyclic dependency graph; missing completion evidence fails validation.</x:v>
+      </x:c>
       <x:c r="M11" s="23" t="str"/>
       <x:c r="N11" s="23" t="str">
         <x:v>https://v5ma.github.io/theology-wiki/san-reader.html?page=research-roadmap</x:v>
@@ -1853,7 +1965,9 @@
 theology-wiki/tests/roadmap.test.cjs</x:v>
       </x:c>
       <x:c r="K12" s="30"/>
-      <x:c r="L12" s="28" t="str"/>
+      <x:c r="L12" s="28" t="str">
+        <x:v>All 354 source rows are generated from actual article references and selected anchors; unlinked is never mislabeled unread.</x:v>
+      </x:c>
       <x:c r="M12" s="23" t="str"/>
       <x:c r="N12" s="23" t="str">
         <x:v>https://v5ma.github.io/theology-wiki/san-reader.html?page=source-coverage</x:v>
@@ -1901,7 +2015,9 @@
 theology-wiki/planning/workbook-manifest.json</x:v>
       </x:c>
       <x:c r="K13" s="30"/>
-      <x:c r="L13" s="28" t="str"/>
+      <x:c r="L13" s="28" t="str">
+        <x:v>The workbook includes task dependencies, chapter routes, all source rows and evidence; formula values and source-manifest hashes are checked.</x:v>
+      </x:c>
       <x:c r="M13" s="23" t="str"/>
       <x:c r="N13" s="23" t="str">
         <x:v>https://v5ma.github.io/theology-wiki/san-reader.html?page=research-roadmap</x:v>
@@ -1948,7 +2064,9 @@
 theology-wiki/data/melchizedek-evidence.json</x:v>
       </x:c>
       <x:c r="K14" s="30"/>
-      <x:c r="L14" s="28" t="str"/>
+      <x:c r="L14" s="28" t="str">
+        <x:v>Genesis 14, Psalm 110, Hebrews 7, 11Q13 and Nag Hammadi are compared with passage locators, access scopes, translation credit and original author-turn links.</x:v>
+      </x:c>
       <x:c r="M14" s="23" t="str">
         <x:v>thomas
 teacher-identity</x:v>
@@ -1998,7 +2116,9 @@
         <x:v>theology-wiki/content/developed/daniel-jubilee-and-the-teachers-time.md</x:v>
       </x:c>
       <x:c r="K15" s="30"/>
-      <x:c r="L15" s="28" t="str"/>
+      <x:c r="L15" s="28" t="str">
+        <x:v>Review the separation of the illustrative 176 BCE model from the October 147 BCE appearance and 88 BCE death; assign a specific starting event and distinguish career, office and successor intervals.</x:v>
+      </x:c>
       <x:c r="M15" s="23" t="str">
         <x:v>thomas</x:v>
       </x:c>
@@ -2043,14 +2163,21 @@
       <x:c r="I16" s="23" t="str">
         <x:v>Compare additional passages with exact textual witnesses, differences and alternative transmission paths; do not infer identity from common adjectives.</x:v>
       </x:c>
-      <x:c r="J16" s="23" t="str"/>
+      <x:c r="J16" s="23" t="str">
+        <x:v>editorial/authorial-articles/thomas-sayings-and-transmission.md
+editorial/transmission-evidence.json</x:v>
+      </x:c>
       <x:c r="K16" s="30"/>
-      <x:c r="L16" s="28" t="str"/>
+      <x:c r="L16" s="28" t="str">
+        <x:v>Collate the relevant Greek and Coptic witnesses and review the full Gathercole/James-fragment critical editions. Distinguish institutional succession from changed interpretation; retain unresolved dependence alternatives.</x:v>
+      </x:c>
       <x:c r="M16" s="23" t="str">
         <x:v>thomas</x:v>
       </x:c>
       <x:c r="N16" s="23" t="str">
-        <x:v>https://v5ma.github.io/theology-wiki/san-reader.html?page=tor-thomas-and-gnostic-transmission</x:v>
+        <x:v>https://v5ma.github.io/theology-wiki/san-reader.html?page=tor-thomas-and-gnostic-transmission
+https://v5ma.github.io/theology-wiki/san-reader.html?page=thomas-sayings-and-transmission
+https://v5ma.github.io/theology-wiki/san-reader.html?page=james-and-contested-succession</x:v>
       </x:c>
       <x:c r="O16" s="23" t="n">
         <x:f>IF(E16="Verified output",1,0)</x:f>
@@ -2091,7 +2218,9 @@
       </x:c>
       <x:c r="J17" s="23" t="str"/>
       <x:c r="K17" s="30"/>
-      <x:c r="L17" s="28" t="str"/>
+      <x:c r="L17" s="28" t="str">
+        <x:v>Independently collate 11Q13 II 6-7 and II 18, then verify the full specialist Teacher identification. The new chronology article reviews Williams, not the missing critical-edition work.</x:v>
+      </x:c>
       <x:c r="M17" s="23" t="str">
         <x:v>thomas</x:v>
       </x:c>
@@ -2138,7 +2267,9 @@
       </x:c>
       <x:c r="J18" s="23" t="str"/>
       <x:c r="K18" s="30"/>
-      <x:c r="L18" s="28" t="str"/>
+      <x:c r="L18" s="28" t="str">
+        <x:v>Identify which editions, pages or recordings support the claims acknowledged in the older conversations; later 2026 posts cannot date the 2025 influence.</x:v>
+      </x:c>
       <x:c r="M18" s="23" t="str"/>
       <x:c r="N18" s="23" t="str">
         <x:v>https://v5ma.github.io/theology-wiki/san-reader.html?page=intellectual-debts</x:v>
@@ -2186,7 +2317,9 @@
 theology-wiki/content/developed/onias-egypt-and-priestly-continuity.md</x:v>
       </x:c>
       <x:c r="K19" s="30"/>
-      <x:c r="L19" s="28" t="str"/>
+      <x:c r="L19" s="28" t="str">
+        <x:v>Collate the incompatible Onias accounts and the 343-year duration; investigate actual intermediates from the reported Egyptian priestly network to later Gnostic and Ethiopian traditions.</x:v>
+      </x:c>
       <x:c r="M19" s="23" t="str">
         <x:v>thomas</x:v>
       </x:c>
@@ -2235,13 +2368,16 @@
         <x:v>theology-wiki/data/priestly-evidence.json</x:v>
       </x:c>
       <x:c r="K20" s="30"/>
-      <x:c r="L20" s="28" t="str"/>
+      <x:c r="L20" s="28" t="str">
+        <x:v>Trace an evidenced route from Egyptian priestly carriers to James-centered traditions. Test genealogy, office, mediated priestly imagery and adverse sect classifications separately.</x:v>
+      </x:c>
       <x:c r="M20" s="23" t="str">
         <x:v>teacher-identity</x:v>
       </x:c>
       <x:c r="N20" s="23" t="str">
         <x:v>https://v5ma.github.io/theology-wiki/san-reader.html?page=jesus-teacher-of-righteousness-hypothesis
-https://v5ma.github.io/theology-wiki/san-reader.html?page=onias-egypt-and-priestly-continuity</x:v>
+https://v5ma.github.io/theology-wiki/san-reader.html?page=onias-egypt-and-priestly-continuity
+https://v5ma.github.io/theology-wiki/san-reader.html?page=james-and-contested-succession</x:v>
       </x:c>
       <x:c r="O20" s="23" t="n">
         <x:f>IF(E20="Verified output",1,0)</x:f>
@@ -2282,7 +2418,9 @@
       </x:c>
       <x:c r="J21" s="23" t="str"/>
       <x:c r="K21" s="30"/>
-      <x:c r="L21" s="28" t="str"/>
+      <x:c r="L21" s="28" t="str">
+        <x:v>Confirm the constructive reading and political application; retain the distinction between recorded heaven remarks and inferred motive.</x:v>
+      </x:c>
       <x:c r="M21" s="23" t="str">
         <x:v>inner-model
 will</x:v>
@@ -2329,7 +2467,9 @@
       </x:c>
       <x:c r="J22" s="23" t="str"/>
       <x:c r="K22" s="30"/>
-      <x:c r="L22" s="28" t="str"/>
+      <x:c r="L22" s="28" t="str">
+        <x:v>The existing two worked passages do not substitute for the broad survey the author requested. Add passages and contextual counterexamples.</x:v>
+      </x:c>
       <x:c r="M22" s="23" t="str">
         <x:v>scriptural-axis
 repair-practice</x:v>
@@ -2380,13 +2520,17 @@
 theology-wiki/editorial/computational-foundations.json</x:v>
       </x:c>
       <x:c r="K23" s="30"/>
-      <x:c r="L23" s="28" t="str"/>
+      <x:c r="L23" s="28" t="str">
+        <x:v>Review the TCNR/SIT operational distinctions and the explicit cross-scale bridge. No confirmed new physical signal is claimed.</x:v>
+      </x:c>
       <x:c r="M23" s="23" t="str">
         <x:v>images
 next-inheritors</x:v>
       </x:c>
       <x:c r="N23" s="23" t="str">
-        <x:v>https://v5ma.github.io/theology-wiki/san-reader.html?page=god-and-our-models-of-god</x:v>
+        <x:v>https://v5ma.github.io/theology-wiki/san-reader.html?page=god-and-our-models-of-god
+https://v5ma.github.io/theology-wiki/san-reader.html?page=computational-divine-immanence
+https://v5ma.github.io/theology-wiki/san-reader.html?page=computational-argument-map</x:v>
       </x:c>
       <x:c r="O23" s="23" t="n">
         <x:f>IF(E23="Verified output",1,0)</x:f>
@@ -2427,7 +2571,9 @@
       </x:c>
       <x:c r="J24" s="23" t="str"/>
       <x:c r="K24" s="30"/>
-      <x:c r="L24" s="28" t="str"/>
+      <x:c r="L24" s="28" t="str">
+        <x:v>Confirm the worked example represents the original argument: the moral model is scrutinized as well as used.</x:v>
+      </x:c>
       <x:c r="M24" s="23" t="str">
         <x:v>inner-model</x:v>
       </x:c>
@@ -2473,7 +2619,9 @@
       </x:c>
       <x:c r="J25" s="23" t="str"/>
       <x:c r="K25" s="30"/>
-      <x:c r="L25" s="28" t="str"/>
+      <x:c r="L25" s="28" t="str">
+        <x:v>Recover full original passages and their dates before outcome assessment. Existing recovery leads remain unscored.</x:v>
+      </x:c>
       <x:c r="M25" s="23" t="str">
         <x:v>warnings</x:v>
       </x:c>
@@ -2520,7 +2668,9 @@
       </x:c>
       <x:c r="J26" s="23" t="str"/>
       <x:c r="K26" s="30"/>
-      <x:c r="L26" s="28" t="str"/>
+      <x:c r="L26" s="28" t="str">
+        <x:v>Select Gnostic and non-Gnostic texts with independently justified dates; distinguish grief, just anger, rejection of creation and institutional repair.</x:v>
+      </x:c>
       <x:c r="M26" s="23" t="str">
         <x:v>trauma</x:v>
       </x:c>
@@ -2569,13 +2719,16 @@
         <x:v>theology-wiki/editorial/authorial-articles/flood-inheritance-and-deep-time.md</x:v>
       </x:c>
       <x:c r="K27" s="30"/>
-      <x:c r="L27" s="28" t="str"/>
+      <x:c r="L27" s="28" t="str">
+        <x:v>Extend exact flood-passage mappings and competing transmission accounts; replace illustrative likelihoods only after calibration and dependency review.</x:v>
+      </x:c>
       <x:c r="M27" s="23" t="str">
         <x:v>shared-archive
 continuing</x:v>
       </x:c>
       <x:c r="N27" s="23" t="str">
-        <x:v>https://v5ma.github.io/theology-wiki/san-reader.html?page=sacred-inheritance-and-rival-continuations</x:v>
+        <x:v>https://v5ma.github.io/theology-wiki/san-reader.html?page=sacred-inheritance-and-rival-continuations
+https://v5ma.github.io/theology-wiki/san-reader.html?page=flood-inheritance-and-deep-time</x:v>
       </x:c>
       <x:c r="O27" s="23" t="n">
         <x:f>IF(E27="Verified output",1,0)</x:f>
@@ -2616,7 +2769,9 @@
       </x:c>
       <x:c r="J28" s="23" t="str"/>
       <x:c r="K28" s="30"/>
-      <x:c r="L28" s="28" t="str"/>
+      <x:c r="L28" s="28" t="str">
+        <x:v>Separate the author's teaching proposal from the new editorial question about obligations toward future conscious participants.</x:v>
+      </x:c>
       <x:c r="M28" s="23" t="str">
         <x:v>next-inheritors</x:v>
       </x:c>
@@ -2662,7 +2817,9 @@
       </x:c>
       <x:c r="J29" s="23" t="str"/>
       <x:c r="K29" s="30"/>
-      <x:c r="L29" s="28" t="str"/>
+      <x:c r="L29" s="28" t="str">
+        <x:v>The existing public source seed still calls itself private-first. Confirm its intended editorial status without changing the original file automatically.</x:v>
+      </x:c>
       <x:c r="M29" s="23" t="str">
         <x:v>shared-archive
 continuing</x:v>
@@ -2710,7 +2867,9 @@
       </x:c>
       <x:c r="J30" s="23" t="str"/>
       <x:c r="K30" s="30"/>
-      <x:c r="L30" s="28" t="str"/>
+      <x:c r="L30" s="28" t="str">
+        <x:v>The contents is a proposed argument order, not a finished manuscript. Confirm whether the sequence preserves the breadth of the author's project.</x:v>
+      </x:c>
       <x:c r="M30" s="23" t="str">
         <x:v>shared-archive
 names
@@ -2776,7 +2935,9 @@
 theology-wiki/content/developed/exodus-to-temple-competing-chronologies.md</x:v>
       </x:c>
       <x:c r="K31" s="30"/>
-      <x:c r="L31" s="28" t="str"/>
+      <x:c r="L31" s="28" t="str">
+        <x:v>Every developed article has reviewed claims, original corrections, rejected readings and a scoped list of sources; source linking alone is not a fidelity sign-off.</x:v>
+      </x:c>
       <x:c r="M31" s="23" t="str"/>
       <x:c r="N31" s="23" t="str">
         <x:v>https://v5ma.github.io/theology-wiki/san-reader.html?page=source-coverage</x:v>
@@ -2820,7 +2981,9 @@
       </x:c>
       <x:c r="J32" s="23" t="str"/>
       <x:c r="K32" s="30"/>
-      <x:c r="L32" s="28" t="str"/>
+      <x:c r="L32" s="28" t="str">
+        <x:v>Compare exact textual readings and institutional claims for a selected sacred-center dispute with dates, translations and alternative interpretations.</x:v>
+      </x:c>
       <x:c r="M32" s="23" t="str">
         <x:v>shared-archive</x:v>
       </x:c>
@@ -2867,7 +3030,9 @@
       </x:c>
       <x:c r="J33" s="23" t="str"/>
       <x:c r="K33" s="30"/>
-      <x:c r="L33" s="28" t="str"/>
+      <x:c r="L33" s="28" t="str">
+        <x:v>Preserve dated candidates and whether each is an allegory, institutional role or fulfillment claim; explain what remains stable across versions.</x:v>
+      </x:c>
       <x:c r="M33" s="23" t="str">
         <x:v>beast</x:v>
       </x:c>
@@ -2914,7 +3079,9 @@
       </x:c>
       <x:c r="J34" s="23" t="str"/>
       <x:c r="K34" s="30"/>
-      <x:c r="L34" s="28" t="str"/>
+      <x:c r="L34" s="28" t="str">
+        <x:v>Recovered original predictions, conditions and dates remain immutable; later observations and assessments are separate records. No retroactive threshold is labeled preregistered.</x:v>
+      </x:c>
       <x:c r="M34" s="23" t="str">
         <x:v>warnings</x:v>
       </x:c>
@@ -2961,7 +3128,9 @@
       </x:c>
       <x:c r="J35" s="23" t="str"/>
       <x:c r="K35" s="30"/>
-      <x:c r="L35" s="28" t="str"/>
+      <x:c r="L35" s="28" t="str">
+        <x:v>Each chapter has an argument map, worked sources, competing explanations, attribution, author review and a narrative handoff; no readiness is inferred from word count.</x:v>
+      </x:c>
       <x:c r="M35" s="23" t="str">
         <x:v>shared-archive
 names
@@ -3025,7 +3194,9 @@
       </x:c>
       <x:c r="J36" s="23" t="str"/>
       <x:c r="K36" s="30"/>
-      <x:c r="L36" s="28" t="str"/>
+      <x:c r="L36" s="28" t="str">
+        <x:v>A complete opening chapter develops the inheritance problem and its transition, with author-approved first-person wording and endnotes.</x:v>
+      </x:c>
       <x:c r="M36" s="23" t="str">
         <x:v>shared-archive</x:v>
       </x:c>
@@ -3072,7 +3243,9 @@
       </x:c>
       <x:c r="J37" s="23" t="str"/>
       <x:c r="K37" s="30"/>
-      <x:c r="L37" s="28" t="str"/>
+      <x:c r="L37" s="28" t="str">
+        <x:v>A pinned chapter map produces manuscript text, stable cross-references and endnotes without copying chat boilerplate. No automatic author-approval flag.</x:v>
+      </x:c>
       <x:c r="M37" s="23" t="str"/>
       <x:c r="N37" s="23" t="str">
         <x:v>https://v5ma.github.io/theology-wiki/san-reader.html?page=book-contents</x:v>
@@ -3116,7 +3289,9 @@
       </x:c>
       <x:c r="J38" s="23" t="str"/>
       <x:c r="K38" s="30"/>
-      <x:c r="L38" s="28" t="str"/>
+      <x:c r="L38" s="28" t="str">
+        <x:v>Micah approves the manuscript argument by argument, including qualifications, intellectual debts, version distinctions and original corrections.</x:v>
+      </x:c>
       <x:c r="M38" s="23" t="str"/>
       <x:c r="N38" s="23" t="str">
         <x:v>https://v5ma.github.io/theology-wiki/san-reader.html?page=book-contents</x:v>
@@ -3162,10 +3337,13 @@
       </x:c>
       <x:c r="J39" s="23" t="str"/>
       <x:c r="K39" s="30"/>
-      <x:c r="L39" s="28" t="str"/>
+      <x:c r="L39" s="28" t="str">
+        <x:v>Every scholarly claim has a consulted edition/location; all quotation and image licenses and required credits are checked.</x:v>
+      </x:c>
       <x:c r="M39" s="23" t="str"/>
       <x:c r="N39" s="23" t="str">
-        <x:v>https://v5ma.github.io/theology-wiki/san-reader.html?page=intellectual-debts</x:v>
+        <x:v>https://v5ma.github.io/theology-wiki/san-reader.html?page=intellectual-debts
+https://v5ma.github.io/theology-wiki/san-reader.html?page=image-collection</x:v>
       </x:c>
       <x:c r="O39" s="23" t="n">
         <x:f>IF(E39="Verified output",1,0)</x:f>
@@ -3207,7 +3385,9 @@
       </x:c>
       <x:c r="J40" s="23" t="str"/>
       <x:c r="K40" s="30"/>
-      <x:c r="L40" s="28" t="str"/>
+      <x:c r="L40" s="28" t="str">
+        <x:v>Remove duplication and inconsistent terms without deleting substantive distinctions; maintain a traceable editorial change log.</x:v>
+      </x:c>
       <x:c r="M40" s="23" t="str"/>
       <x:c r="N40" s="23" t="str">
         <x:v>https://v5ma.github.io/theology-wiki/san-reader.html?page=book-contents</x:v>
@@ -3251,7 +3431,9 @@
       </x:c>
       <x:c r="J41" s="23" t="str"/>
       <x:c r="K41" s="30"/>
-      <x:c r="L41" s="28" t="str"/>
+      <x:c r="L41" s="28" t="str">
+        <x:v>Run complete content/browser checks, read every print-layout page, verify links and credits, and archive the exact approved edition.</x:v>
+      </x:c>
       <x:c r="M41" s="23" t="str"/>
       <x:c r="N41" s="23" t="str">
         <x:v>https://v5ma.github.io/theology-wiki/san-reader.html?page=research-roadmap</x:v>
@@ -3296,7 +3478,9 @@
       </x:c>
       <x:c r="J42" s="23" t="str"/>
       <x:c r="K42" s="30"/>
-      <x:c r="L42" s="28" t="str"/>
+      <x:c r="L42" s="28" t="str">
+        <x:v>Publish only after author sign-off, rights and technical checks; pin source versions and maintain a dated errata record.</x:v>
+      </x:c>
       <x:c r="M42" s="23" t="str"/>
       <x:c r="N42" s="23" t="str">
         <x:v>https://v5ma.github.io/theology-wiki/san-reader.html?page=book-contents</x:v>
@@ -3333,7 +3517,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5ddcef50f9bd403f"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd1c39240d74644ab"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3351,32 +3535,32 @@
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="36" customHeight="1">
-      <x:c r="A1" s="5" t="str">
+      <x:c r="A1" s="69" t="str">
         <x:v>Theology | Dependency edges</x:v>
       </x:c>
-      <x:c r="B1" s="5"/>
-      <x:c r="C1" s="5"/>
-      <x:c r="D1" s="5"/>
-      <x:c r="E1" s="5"/>
-      <x:c r="F1" s="5"/>
+      <x:c r="B1" s="69"/>
+      <x:c r="C1" s="69"/>
+      <x:c r="D1" s="69"/>
+      <x:c r="E1" s="69"/>
+      <x:c r="F1" s="69"/>
     </x:row>
     <x:row r="2" ht="22" customHeight="1">
-      <x:c r="A2" s="10" t="str">
+      <x:c r="A2" s="71" t="str">
         <x:v>Each row is a work-order dependency. It is not a logical entailment between theological claims. Status and satisfaction recalculate from Checklist.</x:v>
       </x:c>
-      <x:c r="B2" s="10"/>
-      <x:c r="C2" s="10"/>
-      <x:c r="D2" s="10"/>
-      <x:c r="E2" s="10"/>
-      <x:c r="F2" s="10"/>
+      <x:c r="B2" s="71"/>
+      <x:c r="C2" s="71"/>
+      <x:c r="D2" s="71"/>
+      <x:c r="E2" s="71"/>
+      <x:c r="F2" s="71"/>
     </x:row>
     <x:row r="3" ht="22" customHeight="1">
-      <x:c r="A3" s="10"/>
-      <x:c r="B3" s="10"/>
-      <x:c r="C3" s="10"/>
-      <x:c r="D3" s="10"/>
-      <x:c r="E3" s="10"/>
-      <x:c r="F3" s="10"/>
+      <x:c r="A3" s="71"/>
+      <x:c r="B3" s="71"/>
+      <x:c r="C3" s="71"/>
+      <x:c r="D3" s="71"/>
+      <x:c r="E3" s="71"/>
+      <x:c r="F3" s="71"/>
     </x:row>
     <x:row r="4">
       <x:c r="A4" s="2"/>
@@ -3387,8 +3571,8 @@
       <x:c r="F4" s="2"/>
     </x:row>
     <x:row r="5" ht="20" customHeight="1">
-      <x:c r="A5" s="14" t="str">
-        <x:v>Snapshot 2026-09-05 | 2026.09.05-atlas-1 | Shared plan: theology-wiki/editorial/roadmap.json</x:v>
+      <x:c r="A5" s="72" t="str">
+        <x:v>Content edition: 2026.09.06-james-transmission-1</x:v>
       </x:c>
       <x:c r="B5" s="14"/>
       <x:c r="C5" s="14"/>
@@ -4392,7 +4576,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R276491e41745444c"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R035e1f1565db42d6"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4415,47 +4599,47 @@
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="36" customHeight="1">
-      <x:c r="A1" s="5" t="str">
+      <x:c r="A1" s="69" t="str">
         <x:v>Theology | Proposed book sequence</x:v>
       </x:c>
-      <x:c r="B1" s="5"/>
-      <x:c r="C1" s="5"/>
-      <x:c r="D1" s="5"/>
-      <x:c r="E1" s="5"/>
-      <x:c r="F1" s="5"/>
-      <x:c r="G1" s="5"/>
-      <x:c r="H1" s="5"/>
-      <x:c r="I1" s="5"/>
-      <x:c r="J1" s="5"/>
-      <x:c r="K1" s="5"/>
+      <x:c r="B1" s="69"/>
+      <x:c r="C1" s="69"/>
+      <x:c r="D1" s="69"/>
+      <x:c r="E1" s="69"/>
+      <x:c r="F1" s="69"/>
+      <x:c r="G1" s="69"/>
+      <x:c r="H1" s="69"/>
+      <x:c r="I1" s="69"/>
+      <x:c r="J1" s="69"/>
+      <x:c r="K1" s="69"/>
     </x:row>
     <x:row r="2" ht="22" customHeight="1">
-      <x:c r="A2" s="10" t="str">
+      <x:c r="A2" s="71" t="str">
         <x:v>Seventeen routes in five movements are not completed manuscript chapters. Source counts measure recorded references; author approval must be recorded separately.</x:v>
       </x:c>
-      <x:c r="B2" s="10"/>
-      <x:c r="C2" s="10"/>
-      <x:c r="D2" s="10"/>
-      <x:c r="E2" s="10"/>
-      <x:c r="F2" s="10"/>
-      <x:c r="G2" s="10"/>
-      <x:c r="H2" s="10"/>
-      <x:c r="I2" s="10"/>
-      <x:c r="J2" s="10"/>
-      <x:c r="K2" s="10"/>
+      <x:c r="B2" s="71"/>
+      <x:c r="C2" s="71"/>
+      <x:c r="D2" s="71"/>
+      <x:c r="E2" s="71"/>
+      <x:c r="F2" s="71"/>
+      <x:c r="G2" s="71"/>
+      <x:c r="H2" s="71"/>
+      <x:c r="I2" s="71"/>
+      <x:c r="J2" s="71"/>
+      <x:c r="K2" s="71"/>
     </x:row>
     <x:row r="3" ht="22" customHeight="1">
-      <x:c r="A3" s="10"/>
-      <x:c r="B3" s="10"/>
-      <x:c r="C3" s="10"/>
-      <x:c r="D3" s="10"/>
-      <x:c r="E3" s="10"/>
-      <x:c r="F3" s="10"/>
-      <x:c r="G3" s="10"/>
-      <x:c r="H3" s="10"/>
-      <x:c r="I3" s="10"/>
-      <x:c r="J3" s="10"/>
-      <x:c r="K3" s="10"/>
+      <x:c r="A3" s="71"/>
+      <x:c r="B3" s="71"/>
+      <x:c r="C3" s="71"/>
+      <x:c r="D3" s="71"/>
+      <x:c r="E3" s="71"/>
+      <x:c r="F3" s="71"/>
+      <x:c r="G3" s="71"/>
+      <x:c r="H3" s="71"/>
+      <x:c r="I3" s="71"/>
+      <x:c r="J3" s="71"/>
+      <x:c r="K3" s="71"/>
     </x:row>
     <x:row r="4">
       <x:c r="A4" s="2"/>
@@ -4471,8 +4655,8 @@
       <x:c r="K4" s="2"/>
     </x:row>
     <x:row r="5" ht="20" customHeight="1">
-      <x:c r="A5" s="14" t="str">
-        <x:v>Snapshot 2026-09-05 | 2026.09.05-atlas-1 | Shared plan: theology-wiki/editorial/roadmap.json</x:v>
+      <x:c r="A5" s="72" t="str">
+        <x:v>Content edition: 2026.09.06-james-transmission-1</x:v>
       </x:c>
       <x:c r="B5" s="14"/>
       <x:c r="C5" s="14"/>
@@ -4666,17 +4850,21 @@
       </x:c>
       <x:c r="E10" s="23" t="str">
         <x:v>jesus-teacher-of-righteousness-hypothesis
-daniel-jubilee-and-the-teachers-time</x:v>
+daniel-jubilee-and-the-teachers-time
+james-and-contested-succession</x:v>
       </x:c>
       <x:c r="F10" s="23" t="str">
         <x:v>teacher-of-righteousness-vs-gnostic-jesus
 pilate-life-timeline
 daniel-and-teacher-of-righteousness
-ai-re-dates-dead-sea-scrolls</x:v>
+ai-re-dates-dead-sea-scrolls
+james-the-just-analysis
+paul-vs-james-movement
+jesus-and-biblical-figures</x:v>
       </x:c>
       <x:c r="G10" s="23" t="n">
         <x:f>IF(F10="",0,LEN(F10)-LEN(SUBSTITUTE(F10,CHAR(10),""))+1)</x:f>
-        <x:v>4</x:v>
+        <x:v>7</x:v>
       </x:c>
       <x:c r="H10" s="23" t="str">
         <x:v>melchizedek-first-pass
@@ -4712,7 +4900,9 @@
         <x:v>tor-thomas-and-gnostic-transmission
 melchizedek-priesthood-and-transmission
 manuscripts-movements-and-survival
-onias-egypt-and-priestly-continuity</x:v>
+onias-egypt-and-priestly-continuity
+james-and-contested-succession
+thomas-sayings-and-transmission</x:v>
       </x:c>
       <x:c r="F11" s="23" t="str">
         <x:v>teacher-of-righteousness-vs-gnostic-jesus
@@ -4720,11 +4910,13 @@
 daniel-and-teacher-of-righteousness
 paul-vs-james-movement
 who-was-josepheous
-jewish-apocalyptic-repair-timeline</x:v>
+jewish-apocalyptic-repair-timeline
+james-the-just-analysis
+jesus-and-biblical-figures</x:v>
       </x:c>
       <x:c r="G11" s="23" t="n">
         <x:f>IF(F11="",0,LEN(F11)-LEN(SUBSTITUTE(F11,CHAR(10),""))+1)</x:f>
-        <x:v>6</x:v>
+        <x:v>8</x:v>
       </x:c>
       <x:c r="H11" s="23" t="str">
         <x:v>melchizedek-first-pass
@@ -4850,18 +5042,21 @@
         <x:v>Not assessed as a manuscript chapter</x:v>
       </x:c>
       <x:c r="E14" s="23" t="str">
-        <x:v>cognitive-gnosticism</x:v>
+        <x:v>cognitive-gnosticism
+thomas-sayings-and-transmission</x:v>
       </x:c>
       <x:c r="F14" s="23" t="str">
         <x:v>cognitive-gnosticism-jesus-vs-gnostic-jesus
 publishing-cognitive-gnosticism-first
 antichrist-spiritual-inversion
 teacher-of-righteousness-vs-gnostic-jesus
-faith-as-vibration-concept</x:v>
+faith-as-vibration-concept
+jesus-and-biblical-figures
+ai-re-dates-dead-sea-scrolls</x:v>
       </x:c>
       <x:c r="G14" s="23" t="n">
         <x:f>IF(F14="",0,LEN(F14)-LEN(SUBSTITUTE(F14,CHAR(10),""))+1)</x:f>
-        <x:v>5</x:v>
+        <x:v>7</x:v>
       </x:c>
       <x:c r="H14" s="23" t="str">
         <x:v>chapter-arc
@@ -4893,7 +5088,8 @@
       <x:c r="E15" s="23" t="str">
         <x:v>christ-as-an-inner-model
 divine-will-and-self-authorizing-power
-inner-formation-texts-and-material-witnesses</x:v>
+inner-formation-texts-and-material-witnesses
+thomas-sayings-and-transmission</x:v>
       </x:c>
       <x:c r="F15" s="23" t="str">
         <x:v>cognitive-gnosticism-jesus-vs-gnostic-jesus
@@ -4902,11 +5098,12 @@
 samuel-vs-micah-divide
 resurrection-debate-in-christianity
 agi-religious-framework
-ai-re-dates-dead-sea-scrolls</x:v>
+ai-re-dates-dead-sea-scrolls
+jesus-and-biblical-figures</x:v>
       </x:c>
       <x:c r="G15" s="23" t="n">
         <x:f>IF(F15="",0,LEN(F15)-LEN(SUBSTITUTE(F15,CHAR(10),""))+1)</x:f>
-        <x:v>7</x:v>
+        <x:v>8</x:v>
       </x:c>
       <x:c r="H15" s="23" t="str">
         <x:v>will
@@ -5280,7 +5477,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1cf0cab678f2406c"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5a5b919f591741a2"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5306,56 +5503,56 @@
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="36" customHeight="1">
-      <x:c r="A1" s="5" t="str">
+      <x:c r="A1" s="69" t="str">
         <x:v>Theology | Every preserved conversation</x:v>
       </x:c>
-      <x:c r="B1" s="5"/>
-      <x:c r="C1" s="5"/>
-      <x:c r="D1" s="5"/>
-      <x:c r="E1" s="5"/>
-      <x:c r="F1" s="5"/>
-      <x:c r="G1" s="5"/>
-      <x:c r="H1" s="5"/>
-      <x:c r="I1" s="5"/>
-      <x:c r="J1" s="5"/>
-      <x:c r="K1" s="5"/>
-      <x:c r="L1" s="5"/>
-      <x:c r="M1" s="5"/>
-      <x:c r="N1" s="5"/>
+      <x:c r="B1" s="69"/>
+      <x:c r="C1" s="69"/>
+      <x:c r="D1" s="69"/>
+      <x:c r="E1" s="69"/>
+      <x:c r="F1" s="69"/>
+      <x:c r="G1" s="69"/>
+      <x:c r="H1" s="69"/>
+      <x:c r="I1" s="69"/>
+      <x:c r="J1" s="69"/>
+      <x:c r="K1" s="69"/>
+      <x:c r="L1" s="69"/>
+      <x:c r="M1" s="69"/>
+      <x:c r="N1" s="69"/>
     </x:row>
     <x:row r="2" ht="22" customHeight="1">
-      <x:c r="A2" s="10" t="str">
+      <x:c r="A2" s="71" t="str">
         <x:v>Coverage means recorded links and selected source-turn anchors. It does not measure how much has been read, quality, originality, completeness, or author approval. Export-start dates do not date every later turn. Export-start date is not a date assigned to every later turn.</x:v>
       </x:c>
-      <x:c r="B2" s="10"/>
-      <x:c r="C2" s="10"/>
-      <x:c r="D2" s="10"/>
-      <x:c r="E2" s="10"/>
-      <x:c r="F2" s="10"/>
-      <x:c r="G2" s="10"/>
-      <x:c r="H2" s="10"/>
-      <x:c r="I2" s="10"/>
-      <x:c r="J2" s="10"/>
-      <x:c r="K2" s="10"/>
-      <x:c r="L2" s="10"/>
-      <x:c r="M2" s="10"/>
-      <x:c r="N2" s="10"/>
+      <x:c r="B2" s="71"/>
+      <x:c r="C2" s="71"/>
+      <x:c r="D2" s="71"/>
+      <x:c r="E2" s="71"/>
+      <x:c r="F2" s="71"/>
+      <x:c r="G2" s="71"/>
+      <x:c r="H2" s="71"/>
+      <x:c r="I2" s="71"/>
+      <x:c r="J2" s="71"/>
+      <x:c r="K2" s="71"/>
+      <x:c r="L2" s="71"/>
+      <x:c r="M2" s="71"/>
+      <x:c r="N2" s="71"/>
     </x:row>
     <x:row r="3" ht="22" customHeight="1">
-      <x:c r="A3" s="10"/>
-      <x:c r="B3" s="10"/>
-      <x:c r="C3" s="10"/>
-      <x:c r="D3" s="10"/>
-      <x:c r="E3" s="10"/>
-      <x:c r="F3" s="10"/>
-      <x:c r="G3" s="10"/>
-      <x:c r="H3" s="10"/>
-      <x:c r="I3" s="10"/>
-      <x:c r="J3" s="10"/>
-      <x:c r="K3" s="10"/>
-      <x:c r="L3" s="10"/>
-      <x:c r="M3" s="10"/>
-      <x:c r="N3" s="10"/>
+      <x:c r="A3" s="71"/>
+      <x:c r="B3" s="71"/>
+      <x:c r="C3" s="71"/>
+      <x:c r="D3" s="71"/>
+      <x:c r="E3" s="71"/>
+      <x:c r="F3" s="71"/>
+      <x:c r="G3" s="71"/>
+      <x:c r="H3" s="71"/>
+      <x:c r="I3" s="71"/>
+      <x:c r="J3" s="71"/>
+      <x:c r="K3" s="71"/>
+      <x:c r="L3" s="71"/>
+      <x:c r="M3" s="71"/>
+      <x:c r="N3" s="71"/>
     </x:row>
     <x:row r="4">
       <x:c r="A4" s="2"/>
@@ -5374,8 +5571,8 @@
       <x:c r="N4" s="2"/>
     </x:row>
     <x:row r="5" ht="20" customHeight="1">
-      <x:c r="A5" s="14" t="str">
-        <x:v>Snapshot 2026-09-05 | 2026.09.05-atlas-1 | Shared plan: theology-wiki/editorial/roadmap.json</x:v>
+      <x:c r="A5" s="72" t="str">
+        <x:v>Content edition: 2026.09.06-james-transmission-1</x:v>
       </x:c>
       <x:c r="B5" s="14"/>
       <x:c r="C5" s="14"/>
@@ -5832,11 +6029,13 @@
 manuscripts-movements-and-survival
 inner-formation-texts-and-material-witnesses
 daniel-jubilee-and-the-teachers-time
-onias-egypt-and-priestly-continuity</x:v>
+onias-egypt-and-priestly-continuity
+james-and-contested-succession
+thomas-sayings-and-transmission</x:v>
       </x:c>
       <x:c r="F16" s="23" t="n">
         <x:f>IF(E16="",0,LEN(E16)-LEN(SUBSTITUTE(E16,CHAR(10),""))+1)</x:f>
-        <x:v>8</x:v>
+        <x:v>10</x:v>
       </x:c>
       <x:c r="G16" s="23" t="str">
         <x:v>Turn 22
@@ -5855,6 +6054,7 @@
 teacher-identity
 thomas
 trauma
+gnosis
 inner-model
 continuing</x:v>
       </x:c>
@@ -12523,19 +12723,24 @@
       <x:c r="D181" s="23" t="n">
         <x:v>4</x:v>
       </x:c>
-      <x:c r="E181" s="23" t="str"/>
+      <x:c r="E181" s="23" t="str">
+        <x:v>james-and-contested-succession</x:v>
+      </x:c>
       <x:c r="F181" s="23" t="n">
         <x:f>IF(E181="",0,LEN(E181)-LEN(SUBSTITUTE(E181,CHAR(10),""))+1)</x:f>
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="G181" s="23" t="str"/>
       <x:c r="H181" s="23" t="n">
         <x:f>IF(G181="",0,LEN(G181&amp;"")-LEN(SUBSTITUTE(G181&amp;"",CHAR(10),""))+1)</x:f>
         <x:v>0</x:v>
       </x:c>
-      <x:c r="I181" s="23" t="str"/>
+      <x:c r="I181" s="23" t="str">
+        <x:v>teacher-identity
+thomas</x:v>
+      </x:c>
       <x:c r="J181" s="23" t="str">
-        <x:v>No developed-article link recorded</x:v>
+        <x:v>Linked to developed article</x:v>
       </x:c>
       <x:c r="K181" s="23" t="str">
         <x:v>Not inferred</x:v>
@@ -12603,19 +12808,27 @@
       <x:c r="D183" s="23" t="n">
         <x:v>10</x:v>
       </x:c>
-      <x:c r="E183" s="23" t="str"/>
+      <x:c r="E183" s="23" t="str">
+        <x:v>james-and-contested-succession
+thomas-sayings-and-transmission</x:v>
+      </x:c>
       <x:c r="F183" s="23" t="n">
         <x:f>IF(E183="",0,LEN(E183)-LEN(SUBSTITUTE(E183,CHAR(10),""))+1)</x:f>
-        <x:v>0</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="G183" s="23" t="str"/>
       <x:c r="H183" s="23" t="n">
         <x:f>IF(G183="",0,LEN(G183&amp;"")-LEN(SUBSTITUTE(G183&amp;"",CHAR(10),""))+1)</x:f>
         <x:v>0</x:v>
       </x:c>
-      <x:c r="I183" s="23" t="str"/>
+      <x:c r="I183" s="23" t="str">
+        <x:v>teacher-identity
+thomas
+gnosis
+inner-model</x:v>
+      </x:c>
       <x:c r="J183" s="23" t="str">
-        <x:v>No developed-article link recorded</x:v>
+        <x:v>Linked to developed article</x:v>
       </x:c>
       <x:c r="K183" s="23" t="str">
         <x:v>Not inferred</x:v>
@@ -15562,11 +15775,12 @@
       </x:c>
       <x:c r="E256" s="23" t="str">
         <x:v>sacred-inheritance-and-rival-continuations
-tor-thomas-and-gnostic-transmission</x:v>
+tor-thomas-and-gnostic-transmission
+james-and-contested-succession</x:v>
       </x:c>
       <x:c r="F256" s="23" t="n">
         <x:f>IF(E256="",0,LEN(E256)-LEN(SUBSTITUTE(E256,CHAR(10),""))+1)</x:f>
-        <x:v>2</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="G256" s="23" t="str">
         <x:v>Turn 1</x:v>
@@ -15577,6 +15791,7 @@
       </x:c>
       <x:c r="I256" s="23" t="str">
         <x:v>shared-archive
+teacher-identity
 thomas
 continuing</x:v>
       </x:c>
@@ -19835,7 +20050,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6b02113a87af4b14"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb1209acb76d3430a"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -19845,48 +20060,56 @@
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
     <x:col min="1" max="1" width="30" hidden="0" customWidth="1"/>
-    <x:col min="2" max="2" width="48" hidden="0" customWidth="1"/>
-    <x:col min="3" max="3" width="46" hidden="0" customWidth="1"/>
-    <x:col min="4" max="4" width="54" hidden="0" customWidth="1"/>
-    <x:col min="5" max="5" width="56" hidden="0" customWidth="1"/>
-    <x:col min="6" max="6" width="55" hidden="0" customWidth="1"/>
-    <x:col min="7" max="7" width="62" hidden="0" customWidth="1"/>
-    <x:col min="8" max="8" width="72" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="30" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="40" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="26" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="40" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="32" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="40" hidden="0" customWidth="1"/>
+    <x:col min="8" max="8" width="35" hidden="0" customWidth="1"/>
+    <x:col min="9" max="9" width="29" hidden="0" customWidth="1"/>
+    <x:col min="10" max="10" width="40" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="36" customHeight="1">
-      <x:c r="A1" s="5" t="str">
-        <x:v>Theology | First Melchizedek comparison</x:v>
-      </x:c>
-      <x:c r="B1" s="5"/>
-      <x:c r="C1" s="5"/>
-      <x:c r="D1" s="5"/>
-      <x:c r="E1" s="5"/>
-      <x:c r="F1" s="5"/>
-      <x:c r="G1" s="5"/>
-      <x:c r="H1" s="5"/>
+      <x:c r="A1" s="69" t="str">
+        <x:v>Theology | Passage evidence and comparison</x:v>
+      </x:c>
+      <x:c r="B1" s="69"/>
+      <x:c r="C1" s="69"/>
+      <x:c r="D1" s="69"/>
+      <x:c r="E1" s="69"/>
+      <x:c r="F1" s="69"/>
+      <x:c r="G1" s="69"/>
+      <x:c r="H1" s="69"/>
+      <x:c r="I1" s="74"/>
+      <x:c r="J1" s="74"/>
     </x:row>
     <x:row r="2" ht="22" customHeight="1">
-      <x:c r="A2" s="10" t="str">
-        <x:v>These passage locators and access notes support a first comparison, not proof of individual identity or a completed institutional-transmission study.</x:v>
-      </x:c>
-      <x:c r="B2" s="10"/>
-      <x:c r="C2" s="10"/>
-      <x:c r="D2" s="10"/>
-      <x:c r="E2" s="10"/>
-      <x:c r="F2" s="10"/>
-      <x:c r="G2" s="10"/>
-      <x:c r="H2" s="10"/>
+      <x:c r="A2" s="71" t="str">
+        <x:v>Preserved Melchizedek records plus the 30-claim comparison. A source contribution, interpretive boundary and next question are not a probability score.</x:v>
+      </x:c>
+      <x:c r="B2" s="71"/>
+      <x:c r="C2" s="71"/>
+      <x:c r="D2" s="71"/>
+      <x:c r="E2" s="71"/>
+      <x:c r="F2" s="71"/>
+      <x:c r="G2" s="71"/>
+      <x:c r="H2" s="71"/>
+      <x:c r="I2" s="74"/>
+      <x:c r="J2" s="74"/>
     </x:row>
     <x:row r="3" ht="22" customHeight="1">
-      <x:c r="A3" s="10"/>
-      <x:c r="B3" s="10"/>
-      <x:c r="C3" s="10"/>
-      <x:c r="D3" s="10"/>
-      <x:c r="E3" s="10"/>
-      <x:c r="F3" s="10"/>
-      <x:c r="G3" s="10"/>
-      <x:c r="H3" s="10"/>
+      <x:c r="A3" s="71"/>
+      <x:c r="B3" s="71"/>
+      <x:c r="C3" s="71"/>
+      <x:c r="D3" s="71"/>
+      <x:c r="E3" s="71"/>
+      <x:c r="F3" s="71"/>
+      <x:c r="G3" s="71"/>
+      <x:c r="H3" s="71"/>
+      <x:c r="I3" s="74"/>
+      <x:c r="J3" s="74"/>
     </x:row>
     <x:row r="4">
       <x:c r="A4" s="2"/>
@@ -19899,8 +20122,8 @@
       <x:c r="H4" s="2"/>
     </x:row>
     <x:row r="5" ht="20" customHeight="1">
-      <x:c r="A5" s="14" t="str">
-        <x:v>Snapshot 2026-09-05 | 2026.09.05-atlas-1 | Shared plan: theology-wiki/editorial/roadmap.json</x:v>
+      <x:c r="A5" s="72" t="str">
+        <x:v>Content edition: 2026.09.06-james-transmission-1</x:v>
       </x:c>
       <x:c r="B5" s="14"/>
       <x:c r="C5" s="14"/>
@@ -19911,159 +20134,1135 @@
       <x:c r="H5" s="14"/>
     </x:row>
     <x:row r="6" ht="32" customHeight="1">
-      <x:c r="A6" s="18" t="str">
+      <x:c r="A6" s="79" t="str">
         <x:v>Witness / text</x:v>
       </x:c>
-      <x:c r="B6" s="18" t="str">
+      <x:c r="B6" s="79" t="str">
         <x:v>Passage locator</x:v>
       </x:c>
-      <x:c r="C6" s="18" t="str">
+      <x:c r="C6" s="79" t="str">
         <x:v>Role in this reading</x:v>
       </x:c>
-      <x:c r="D6" s="18" t="str">
+      <x:c r="D6" s="79" t="str">
         <x:v>Comparison</x:v>
       </x:c>
-      <x:c r="E6" s="18" t="str">
+      <x:c r="E6" s="79" t="str">
         <x:v>What is not established</x:v>
       </x:c>
-      <x:c r="F6" s="18" t="str">
+      <x:c r="F6" s="79" t="str">
         <x:v>Source / translator</x:v>
       </x:c>
-      <x:c r="G6" s="18" t="str">
+      <x:c r="G6" s="79" t="str">
         <x:v>Access scope</x:v>
       </x:c>
-      <x:c r="H6" s="18" t="str">
+      <x:c r="H6" s="79" t="str">
         <x:v>Source URL</x:v>
       </x:c>
-    </x:row>
-    <x:row r="7" ht="64" customHeight="1">
-      <x:c r="A7" s="23" t="str">
+      <x:c r="I6" s="82" t="str">
+        <x:v>Surviving channel / ID</x:v>
+      </x:c>
+      <x:c r="J6" s="82" t="str">
+        <x:v>Next investigation</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="7" ht="120" customHeight="1">
+      <x:c r="A7" s="77" t="str">
         <x:v>Genesis encounter</x:v>
       </x:c>
-      <x:c r="B7" s="23" t="str">
+      <x:c r="B7" s="77" t="str">
         <x:v>Genesis 14:18-20</x:v>
       </x:c>
-      <x:c r="C7" s="23" t="str">
+      <x:c r="C7" s="77" t="str">
         <x:v>King-priest who blesses Abram and receives a tithe.</x:v>
       </x:c>
-      <x:c r="D7" s="23" t="str">
+      <x:c r="D7" s="77" t="str">
         <x:v>Recognition of sacred authority is narrated before later explanations of institutional descent.</x:v>
       </x:c>
-      <x:c r="E7" s="23" t="str">
+      <x:c r="E7" s="77" t="str">
         <x:v>The passage does not supply an Aaronic or Zadokite genealogy or a transmission route to Qumran.</x:v>
       </x:c>
-      <x:c r="F7" s="23" t="str">
+      <x:c r="F7" s="77" t="str">
         <x:v>Genesis 14:18-20, World English Bible</x:v>
       </x:c>
-      <x:c r="G7" s="23" t="str">
+      <x:c r="G7" s="77" t="str">
         <x:v>Primary chapter consulted. The encounter, blessing and tithe are kept separate from later lineage claims.</x:v>
       </x:c>
-      <x:c r="H7" s="23" t="str">
+      <x:c r="H7" s="77" t="str">
         <x:v>https://ebible.org/engwebp/GEN14.htm</x:v>
       </x:c>
-    </x:row>
-    <x:row r="8" ht="64" customHeight="1">
-      <x:c r="A8" s="23" t="str">
+      <x:c r="I7" s="83"/>
+      <x:c r="J7" s="83"/>
+    </x:row>
+    <x:row r="8" ht="120" customHeight="1">
+      <x:c r="A8" s="77" t="str">
         <x:v>Royal priestly address</x:v>
       </x:c>
-      <x:c r="B8" s="23" t="str">
+      <x:c r="B8" s="77" t="str">
         <x:v>Psalm 110:1-7, especially verse 4</x:v>
       </x:c>
-      <x:c r="C8" s="23" t="str">
+      <x:c r="C8" s="77" t="str">
         <x:v>An enduring priestly appointment in a royal and judicial setting.</x:v>
       </x:c>
-      <x:c r="D8" s="23" t="str">
+      <x:c r="D8" s="77" t="str">
         <x:v>The figure authorizes a role; the surrounding enemy/judgment language must not be omitted.</x:v>
       </x:c>
-      <x:c r="E8" s="23" t="str">
+      <x:c r="E8" s="77" t="str">
         <x:v>A later reading of the royal address is not automatically the original setting of composition.</x:v>
       </x:c>
-      <x:c r="F8" s="23" t="str">
+      <x:c r="F8" s="77" t="str">
         <x:v>Psalm 110, World English Bible</x:v>
       </x:c>
-      <x:c r="G8" s="23" t="str">
+      <x:c r="G8" s="77" t="str">
         <x:v>Primary psalm consulted, especially verses 1-7. Royal and judicial language is retained alongside the priestly address.</x:v>
       </x:c>
-      <x:c r="H8" s="23" t="str">
+      <x:c r="H8" s="77" t="str">
         <x:v>https://ebible.org/engwebp/PSA110.htm</x:v>
       </x:c>
-    </x:row>
-    <x:row r="9" ht="64" customHeight="1">
-      <x:c r="A9" s="23" t="str">
+      <x:c r="I8" s="83"/>
+      <x:c r="J8" s="83"/>
+    </x:row>
+    <x:row r="9" ht="120" customHeight="1">
+      <x:c r="A9" s="77" t="str">
         <x:v>11QMelchizedek</x:v>
       </x:c>
-      <x:c r="B9" s="23" t="str">
+      <x:c r="B9" s="77" t="str">
         <x:v>11Q13 column II, lines 2-9 and 13, through Williams 2023</x:v>
       </x:c>
-      <x:c r="C9" s="23" t="str">
+      <x:c r="C9" s="77" t="str">
         <x:v>Release, restoration and atonement in the consulted scholarly reading.</x:v>
       </x:c>
-      <x:c r="D9" s="23" t="str">
+      <x:c r="D9" s="77" t="str">
         <x:v>Williams argues for an active subject in II 6 rather than an indefinite rendering; this affects the distribution of authority.</x:v>
       </x:c>
-      <x:c r="E9" s="23" t="str">
+      <x:c r="E9" s="77" t="str">
         <x:v>This reading is disputed. Access to a translation and argument does not constitute independent collation of the damaged manuscript.</x:v>
       </x:c>
-      <x:c r="F9" s="23" t="str">
+      <x:c r="F9" s="77" t="str">
         <x:v>Logan Williams (2023), Melchizedek, the Son of Man, and Eschatological Jubilee</x:v>
       </x:c>
-      <x:c r="G9" s="23" t="str">
+      <x:c r="G9" s="77" t="str">
         <x:v>Full-text HTML consulted, particularly the author's translation of 11Q13 II 2-9 and discussion of II 6 and 13. His active-agent reading is distinguished from the critical edition he disputes. The critical edition itself has not been collated in this pass. This is current editorial research, not a recovered author acknowledgment.</x:v>
       </x:c>
-      <x:c r="H9" s="23" t="str">
+      <x:c r="H9" s="77" t="str">
         <x:v>https://journals.sagepub.com/doi/10.1177/0142064X231191176</x:v>
       </x:c>
-    </x:row>
-    <x:row r="10" ht="64" customHeight="1">
-      <x:c r="A10" s="23" t="str">
+      <x:c r="I9" s="83"/>
+      <x:c r="J9" s="83"/>
+    </x:row>
+    <x:row r="10" ht="120" customHeight="1">
+      <x:c r="A10" s="77" t="str">
         <x:v>Continuing priesthood</x:v>
       </x:c>
-      <x:c r="B10" s="23" t="str">
+      <x:c r="B10" s="77" t="str">
         <x:v>Hebrews 7:1-17 and 23-28</x:v>
       </x:c>
-      <x:c r="C10" s="23" t="str">
+      <x:c r="C10" s="77" t="str">
         <x:v>Interpretive superiority and enduring intercession, distinguished from ordinary Levitical qualification.</x:v>
       </x:c>
-      <x:c r="D10" s="23" t="str">
+      <x:c r="D10" s="77" t="str">
         <x:v>The letter uses the inherited figure to reason about a different basis of authority.</x:v>
       </x:c>
-      <x:c r="E10" s="23" t="str">
+      <x:c r="E10" s="77" t="str">
         <x:v>Textual likeness and a continuing role are not evidence that Teacher, James and Jesus are one historical individual.</x:v>
       </x:c>
-      <x:c r="F10" s="23" t="str">
+      <x:c r="F10" s="77" t="str">
         <x:v>Hebrews 7, World English Bible</x:v>
       </x:c>
-      <x:c r="G10" s="23" t="str">
+      <x:c r="G10" s="77" t="str">
         <x:v>Primary chapter consulted, especially verses 1-17 and 23-28. Textual resemblance, descent and continuing priesthood are distinguished.</x:v>
       </x:c>
-      <x:c r="H10" s="23" t="str">
+      <x:c r="H10" s="77" t="str">
         <x:v>https://ebible.org/engwebp/HEB07.htm</x:v>
       </x:c>
-    </x:row>
-    <x:row r="11" ht="64" customHeight="1">
-      <x:c r="A11" s="23" t="str">
+      <x:c r="I10" s="83"/>
+      <x:c r="J10" s="83"/>
+    </x:row>
+    <x:row r="11" ht="120" customHeight="1">
+      <x:c r="A11" s="77" t="str">
         <x:v>Melchizedek tractate</x:v>
       </x:c>
-      <x:c r="B11" s="23" t="str">
+      <x:c r="B11" s="77" t="str">
         <x:v>Nag Hammadi Codex IX,1; online translation, paragraphs on embodiment and the image of the high priest</x:v>
       </x:c>
-      <x:c r="C11" s="23" t="str">
+      <x:c r="C11" s="77" t="str">
         <x:v>Exalted priestly language with ritual participation and explicit embodiment language.</x:v>
       </x:c>
-      <x:c r="D11" s="23" t="str">
+      <x:c r="D11" s="77" t="str">
         <x:v>The anti-docetic passage complicates a universal equation of Gnostic salvation with rejection of the body.</x:v>
       </x:c>
-      <x:c r="E11" s="23" t="str">
+      <x:c r="E11" s="77" t="str">
         <x:v>Extensive gaps prevent an effortless continuous reconstruction. Exact printed page/line citations remain a task.</x:v>
       </x:c>
-      <x:c r="F11" s="23" t="str">
+      <x:c r="F11" s="77" t="str">
         <x:v>Melchizedek, translated by Soren Giversen and Birger A. Pearson</x:v>
       </x:c>
-      <x:c r="G11" s="23" t="str">
+      <x:c r="G11" s="77" t="str">
         <x:v>Online translation retrieved in the indexed full-text result; direct-page retrieval failed. Marked lacunae are retained in the interpretation. The online notice requests published-edition citations for academic work; printed page/line collation remains open. Credit is for a textual source used by this edition, not a claimed personal influence on Micah.</x:v>
       </x:c>
-      <x:c r="H11" s="23" t="str">
+      <x:c r="H11" s="77" t="str">
         <x:v>https://www.gnosis.org/naghamm/melchiz.html</x:v>
+      </x:c>
+      <x:c r="I11" s="83"/>
+      <x:c r="J11" s="83"/>
+    </x:row>
+    <x:row r="12" ht="120" customHeight="1">
+      <x:c r="A12" s="83" t="str">
+        <x:v>James receives and transmits knowledge</x:v>
+      </x:c>
+      <x:c r="B12" s="83" t="str">
+        <x:v>Eusebius 2.1.4, quoting Clement, Hypotyposes 7</x:v>
+      </x:c>
+      <x:c r="C12" s="83" t="str">
+        <x:v>Knowledge is reported as passing through named recipients and subsequent transmitters.</x:v>
+      </x:c>
+      <x:c r="D12" s="83" t="str">
+        <x:v>James and succession</x:v>
+      </x:c>
+      <x:c r="E12" s="83" t="str">
+        <x:v>The complete Hypotyposes is not independently recovered here, and the knowledge is not identified as Thomas.</x:v>
+      </x:c>
+      <x:c r="F12" s="83" t="str">
+        <x:v>Eusebius, Church History 2.1 and 2.23, McGiffert translation</x:v>
+      </x:c>
+      <x:c r="G12" s="83" t="str">
+        <x:v>Consulted the English translation of 2.1.3-4 and 2.23.4-18. Clement and Hegesippus are quoted through Eusebius, not independently recovered complete works. No Greek manuscript collation; narrative details are reported claims, not all independently established events.</x:v>
+      </x:c>
+      <x:c r="H12" s="83" t="str">
+        <x:v>https://www.newadvent.org/fathers/250102.htm</x:v>
+      </x:c>
+      <x:c r="I12" s="83" t="str">
+        <x:v>eusebius / jt-knowledge</x:v>
+      </x:c>
+      <x:c r="J12" s="83" t="str">
+        <x:v>Compare transmitted content and authority without equating knowledge with membership in a later Gnostic school.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="13" ht="120" customHeight="1">
+      <x:c r="A13" s="83" t="str">
+        <x:v>James is portrayed with priestly functions</x:v>
+      </x:c>
+      <x:c r="B13" s="83" t="str">
+        <x:v>Eusebius 2.23.4-7, quoting Hegesippus</x:v>
+      </x:c>
+      <x:c r="C13" s="83" t="str">
+        <x:v>Linen, holy-place access and intercession make priestly representation a concrete comparison.</x:v>
+      </x:c>
+      <x:c r="D13" s="83" t="str">
+        <x:v>James and succession</x:v>
+      </x:c>
+      <x:c r="E13" s="83" t="str">
+        <x:v>The portrayal does not document a Zadokite or Oniad pedigree.</x:v>
+      </x:c>
+      <x:c r="F13" s="83" t="str">
+        <x:v>Eusebius, Church History 2.1 and 2.23, McGiffert translation</x:v>
+      </x:c>
+      <x:c r="G13" s="83" t="str">
+        <x:v>Consulted the English translation of 2.1.3-4 and 2.23.4-18. Clement and Hegesippus are quoted through Eusebius, not independently recovered complete works. No Greek manuscript collation; narrative details are reported claims, not all independently established events.</x:v>
+      </x:c>
+      <x:c r="H13" s="83" t="str">
+        <x:v>https://www.newadvent.org/fathers/250102.htm</x:v>
+      </x:c>
+      <x:c r="I13" s="83" t="str">
+        <x:v>eusebius / jt-priestly-portrait</x:v>
+      </x:c>
+      <x:c r="J13" s="83" t="str">
+        <x:v>Test whether the portrait preserves an office, ritual authority, or retrospective authorization.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="14" ht="120" customHeight="1">
+      <x:c r="A14" s="83" t="str">
+        <x:v>Kinship in the reported succession</x:v>
+      </x:c>
+      <x:c r="B14" s="83" t="str">
+        <x:v>Eusebius 4.22.4-7, quoting Hegesippus</x:v>
+      </x:c>
+      <x:c r="C14" s="83" t="str">
+        <x:v>Symeon is presented as succeeding James with a kinship rationale.</x:v>
+      </x:c>
+      <x:c r="D14" s="83" t="str">
+        <x:v>James and succession</x:v>
+      </x:c>
+      <x:c r="E14" s="83" t="str">
+        <x:v>The same account classifies Essenes as opponents; it is not an unqualified admission of institutional identity.</x:v>
+      </x:c>
+      <x:c r="F14" s="83" t="str">
+        <x:v>Eusebius, Church History 4.22, McGiffert translation</x:v>
+      </x:c>
+      <x:c r="G14" s="83" t="str">
+        <x:v>Consulted 4.22.4-7, including Hegesippus on Symeon, the disputed succession and the classification of Essenes as opponents. The reported kinship and polemical framing remain explicit; no independent reconstruction of the lost Memoirs.</x:v>
+      </x:c>
+      <x:c r="H14" s="83" t="str">
+        <x:v>https://www.newadvent.org/fathers/250104.htm</x:v>
+      </x:c>
+      <x:c r="I14" s="83" t="str">
+        <x:v>eusebius / jt-symeon</x:v>
+      </x:c>
+      <x:c r="J14" s="83" t="str">
+        <x:v>Keep family, office and partisan classifications distinct when testing continuity.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="15" ht="120" customHeight="1">
+      <x:c r="A15" s="83" t="str">
+        <x:v>The particular brother relationship</x:v>
+      </x:c>
+      <x:c r="B15" s="83" t="str">
+        <x:v>Galatians 1:11-20</x:v>
+      </x:c>
+      <x:c r="C15" s="83" t="str">
+        <x:v>Paul singles out James through a relationship to the Lord and recounts a visit after three years.</x:v>
+      </x:c>
+      <x:c r="D15" s="83" t="str">
+        <x:v>James and succession</x:v>
+      </x:c>
+      <x:c r="E15" s="83" t="str">
+        <x:v>Spiritual kinship elsewhere does not automatically explain this particular relationship; the three years do not measure the prior persecution.</x:v>
+      </x:c>
+      <x:c r="F15" s="83" t="str">
+        <x:v>Galatians 1, World English Bible</x:v>
+      </x:c>
+      <x:c r="G15" s="83" t="str">
+        <x:v>Primary text: Paul's account of persecution, revelation, earlier apostles and a visit to Peter and James.</x:v>
+      </x:c>
+      <x:c r="H15" s="83" t="str">
+        <x:v>https://ebible.org/engwebp/GAL01.htm</x:v>
+      </x:c>
+      <x:c r="I15" s="83" t="str">
+        <x:v>galatians / jt-paul-kinship</x:v>
+      </x:c>
+      <x:c r="J15" s="83" t="str">
+        <x:v>Explain the relational wording under the earlier-founder and namesake-successor alternatives.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="16" ht="120" customHeight="1">
+      <x:c r="A16" s="83" t="str">
+        <x:v>Recognition and division of mission</x:v>
+      </x:c>
+      <x:c r="B16" s="83" t="str">
+        <x:v>Galatians 2:1-10</x:v>
+      </x:c>
+      <x:c r="C16" s="83" t="str">
+        <x:v>Paul reports recognition from James, Cephas and John and a division of mission.</x:v>
+      </x:c>
+      <x:c r="D16" s="83" t="str">
+        <x:v>James and succession</x:v>
+      </x:c>
+      <x:c r="E16" s="83" t="str">
+        <x:v>This is Paul's own presentation, not an independent record of every participant's intentions.</x:v>
+      </x:c>
+      <x:c r="F16" s="83" t="str">
+        <x:v>Galatians 2, World English Bible</x:v>
+      </x:c>
+      <x:c r="G16" s="83" t="str">
+        <x:v>Primary text read in full, especially verses 1-10 on an interval, companions and recognized leaders. The passage does not by itself supply an absolute calendar date for the visit.</x:v>
+      </x:c>
+      <x:c r="H16" s="83" t="str">
+        <x:v>https://ebible.org/engwebp/GAL02.htm</x:v>
+      </x:c>
+      <x:c r="I16" s="83" t="str">
+        <x:v>galatians / jt-paul-recognition</x:v>
+      </x:c>
+      <x:c r="J16" s="83" t="str">
+        <x:v>Ask how a rival mission could seek acknowledgment while maintaining a contested program.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="17" ht="120" customHeight="1">
+      <x:c r="A17" s="83" t="str">
+        <x:v>Shared meals and contested authority</x:v>
+      </x:c>
+      <x:c r="B17" s="83" t="str">
+        <x:v>Galatians 2:11-14</x:v>
+      </x:c>
+      <x:c r="C17" s="83" t="str">
+        <x:v>The meal conflict involves arrivals associated with James.</x:v>
+      </x:c>
+      <x:c r="D17" s="83" t="str">
+        <x:v>James and succession</x:v>
+      </x:c>
+      <x:c r="E17" s="83" t="str">
+        <x:v>The paragraph does not explicitly state that James personally ordered the withdrawal.</x:v>
+      </x:c>
+      <x:c r="F17" s="83" t="str">
+        <x:v>Galatians 2, World English Bible</x:v>
+      </x:c>
+      <x:c r="G17" s="83" t="str">
+        <x:v>Primary text read in full, especially verses 1-10 on an interval, companions and recognized leaders. The passage does not by itself supply an absolute calendar date for the visit.</x:v>
+      </x:c>
+      <x:c r="H17" s="83" t="str">
+        <x:v>https://ebible.org/engwebp/GAL02.htm</x:v>
+      </x:c>
+      <x:c r="I17" s="83" t="str">
+        <x:v>galatians / jt-paul-conflict</x:v>
+      </x:c>
+      <x:c r="J17" s="83" t="str">
+        <x:v>Compare association, command and retrospective self-defense rather than attributing an unwritten instruction.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="18" ht="120" customHeight="1">
+      <x:c r="A18" s="83" t="str">
+        <x:v>James in the Festus-Albinus interval</x:v>
+      </x:c>
+      <x:c r="B18" s="83" t="str">
+        <x:v>Antiquities 20.200</x:v>
+      </x:c>
+      <x:c r="C18" s="83" t="str">
+        <x:v>The paragraph provides an administrative interval and identifies James through Jesus called Christ.</x:v>
+      </x:c>
+      <x:c r="D18" s="83" t="str">
+        <x:v>James and succession</x:v>
+      </x:c>
+      <x:c r="E18" s="83" t="str">
+        <x:v>Reading the passage is not a completed authenticity investigation or a license to transfer the death to another person.</x:v>
+      </x:c>
+      <x:c r="F18" s="83" t="str">
+        <x:v>Josephus, Antiquities 20.200, Whiston translation</x:v>
+      </x:c>
+      <x:c r="G18" s="83" t="str">
+        <x:v>Consulted the individual paragraph directly: James, the relational identification, and the Festus-Albinus interval. No new authenticity adjudication, identification of an interpolator, or independent calendar reconstruction is claimed.</x:v>
+      </x:c>
+      <x:c r="H18" s="83" t="str">
+        <x:v>https://lexundria.com/j_aj/20.200/wst</x:v>
+      </x:c>
+      <x:c r="I18" s="83" t="str">
+        <x:v>josephus-antiquities / jt-death</x:v>
+      </x:c>
+      <x:c r="J18" s="83" t="str">
+        <x:v>Specify whether a challenge concerns wording, personal identity, succession or the larger biographical frame.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="19" ht="120" customHeight="1">
+      <x:c r="A19" s="83" t="str">
+        <x:v>Law, Creator and opposition to Paul</x:v>
+      </x:c>
+      <x:c r="B19" s="83" t="str">
+        <x:v>Against Heresies 1.26.2</x:v>
+      </x:c>
+      <x:c r="C19" s="83" t="str">
+        <x:v>The description combines law observance and opposition to Paul with Creator affirmation.</x:v>
+      </x:c>
+      <x:c r="D19" s="83" t="str">
+        <x:v>James and succession</x:v>
+      </x:c>
+      <x:c r="E19" s="83" t="str">
+        <x:v>A hostile external category is not a timeless self-description or automatically a creator-rejecting cosmology.</x:v>
+      </x:c>
+      <x:c r="F19" s="83" t="str">
+        <x:v>Irenaeus, Against Heresies 1.26.2, Roberts-Rambaut translation</x:v>
+      </x:c>
+      <x:c r="G19" s="83" t="str">
+        <x:v>Consulted the translated Ebionite description, including Matthew, opposition to Paul, law observance and Creator affirmation. This is a hostile classifier, not a surviving membership statement from all groups given the name.</x:v>
+      </x:c>
+      <x:c r="H19" s="83" t="str">
+        <x:v>https://www.newadvent.org/fathers/0103126.htm</x:v>
+      </x:c>
+      <x:c r="I19" s="83" t="str">
+        <x:v>irenaeus / jt-ebionites-irenaeus</x:v>
+      </x:c>
+      <x:c r="J19" s="83" t="str">
+        <x:v>Identify which features could persist and which would require a demonstrable transformation.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="20" ht="120" customHeight="1">
+      <x:c r="A20" s="83" t="str">
+        <x:v>Differences inside an inherited label</x:v>
+      </x:c>
+      <x:c r="B20" s="83" t="str">
+        <x:v>Church History 3.27.1-6</x:v>
+      </x:c>
+      <x:c r="C20" s="83" t="str">
+        <x:v>Eusebius distinguishes views among those labeled Ebionites and reports use of a Hebrews gospel.</x:v>
+      </x:c>
+      <x:c r="D20" s="83" t="str">
+        <x:v>James and succession</x:v>
+      </x:c>
+      <x:c r="E20" s="83" t="str">
+        <x:v>The reported gospel title is not automatically an identification of a surviving manuscript or Irenaeus's Matthew.</x:v>
+      </x:c>
+      <x:c r="F20" s="83" t="str">
+        <x:v>Eusebius, Church History 3.27, McGiffert translation</x:v>
+      </x:c>
+      <x:c r="G20" s="83" t="str">
+        <x:v>Consulted chapter 27 on the categories called Ebionites. An external polemical classification with internal distinctions, not an unmediated self-description or catalogue identification of an extant Hebrews gospel.</x:v>
+      </x:c>
+      <x:c r="H20" s="83" t="str">
+        <x:v>https://www.newadvent.org/fathers/250103.htm</x:v>
+      </x:c>
+      <x:c r="I20" s="83" t="str">
+        <x:v>eusebius / jt-ebionites-eusebius</x:v>
+      </x:c>
+      <x:c r="J20" s="83" t="str">
+        <x:v>Compare the classifiers' access and purposes before combining their descriptions.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="21" ht="120" customHeight="1">
+      <x:c r="A21" s="83" t="str">
+        <x:v>James as the communal destination</x:v>
+      </x:c>
+      <x:c r="B21" s="83" t="str">
+        <x:v>Gospel of Thomas 12</x:v>
+      </x:c>
+      <x:c r="C21" s="83" t="str">
+        <x:v>The disciples are directed toward James after Jesus's departure.</x:v>
+      </x:c>
+      <x:c r="D21" s="83" t="str">
+        <x:v>Thomas and formation</x:v>
+      </x:c>
+      <x:c r="E21" s="83" t="str">
+        <x:v>The saying does not supply a calendar date or an explicit ritual of appointing a replacement Christ.</x:v>
+      </x:c>
+      <x:c r="F21" s="83" t="str">
+        <x:v>Gospel of Thomas, translation by Stephen Patterson and Marvin Meyer</x:v>
+      </x:c>
+      <x:c r="G21" s="83" t="str">
+        <x:v>Translation consulted for sayings 1, 3, 12, 13, 39 and 108. The edition uses brief paraphrases and links, not a reproduction of the translation. Translation credit is distinct from an acknowledged influence in the author's older conversations.</x:v>
+      </x:c>
+      <x:c r="H21" s="83" t="str">
+        <x:v>https://www.earlychristianwritings.com/text/thomas-scholars.html</x:v>
+      </x:c>
+      <x:c r="I21" s="83" t="str">
+        <x:v>thomas-coptic / jt-thomas-james</x:v>
+      </x:c>
+      <x:c r="J21" s="83" t="str">
+        <x:v>Compare communal authority with the different authority attributed to Thomas in the next saying.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="22" ht="120" customHeight="1">
+      <x:c r="A22" s="83" t="str">
+        <x:v>Thomas and the private exchange</x:v>
+      </x:c>
+      <x:c r="B22" s="83" t="str">
+        <x:v>Gospel of Thomas 13</x:v>
+      </x:c>
+      <x:c r="C22" s="83" t="str">
+        <x:v>Thomas receives a private exchange and withholds its sayings from the others.</x:v>
+      </x:c>
+      <x:c r="D22" s="83" t="str">
+        <x:v>Thomas and formation</x:v>
+      </x:c>
+      <x:c r="E22" s="83" t="str">
+        <x:v>The passage does not explicitly instruct recruitment of twelve strangers or repeated biographical reenactment.</x:v>
+      </x:c>
+      <x:c r="F22" s="83" t="str">
+        <x:v>Gospel of Thomas, translation by Stephen Patterson and Marvin Meyer</x:v>
+      </x:c>
+      <x:c r="G22" s="83" t="str">
+        <x:v>Translation consulted for sayings 1, 3, 12, 13, 39 and 108. The edition uses brief paraphrases and links, not a reproduction of the translation. Translation credit is distinct from an acknowledged influence in the author's older conversations.</x:v>
+      </x:c>
+      <x:c r="H22" s="83" t="str">
+        <x:v>https://www.earlychristianwritings.com/text/thomas-scholars.html</x:v>
+      </x:c>
+      <x:c r="I22" s="83" t="str">
+        <x:v>thomas-coptic / jt-thomas-private</x:v>
+      </x:c>
+      <x:c r="J22" s="83" t="str">
+        <x:v>State how the succession-through-teaching proposal extends beyond the surviving narrative.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="23" ht="120" customHeight="1">
+      <x:c r="A23" s="83" t="str">
+        <x:v>Interpretation changes the recipient</x:v>
+      </x:c>
+      <x:c r="B23" s="83" t="str">
+        <x:v>Gospel of Thomas 1, 3 and 108</x:v>
+      </x:c>
+      <x:c r="C23" s="83" t="str">
+        <x:v>Life through interpretation, self-knowledge and transformation motivate a formation-oriented reading.</x:v>
+      </x:c>
+      <x:c r="D23" s="83" t="str">
+        <x:v>Thomas and formation</x:v>
+      </x:c>
+      <x:c r="E23" s="83" t="str">
+        <x:v>These translated passages are not measurements or ancient formulations of neural phase dynamics.</x:v>
+      </x:c>
+      <x:c r="F23" s="83" t="str">
+        <x:v>Gospel of Thomas, translation by Stephen Patterson and Marvin Meyer</x:v>
+      </x:c>
+      <x:c r="G23" s="83" t="str">
+        <x:v>Translation consulted for sayings 1, 3, 12, 13, 39 and 108. The edition uses brief paraphrases and links, not a reproduction of the translation. Translation credit is distinct from an acknowledged influence in the author's older conversations.</x:v>
+      </x:c>
+      <x:c r="H23" s="83" t="str">
+        <x:v>https://www.earlychristianwritings.com/text/thomas-scholars.html</x:v>
+      </x:c>
+      <x:c r="I23" s="83" t="str">
+        <x:v>thomas-coptic / jt-thomas-formation</x:v>
+      </x:c>
+      <x:c r="J23" s="83" t="str">
+        <x:v>Distinguish repeated belief from an operative change in perception, motives and choice.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="24" ht="120" customHeight="1">
+      <x:c r="A24" s="83" t="str">
+        <x:v>Blocked access to knowledge in Thomas</x:v>
+      </x:c>
+      <x:c r="B24" s="83" t="str">
+        <x:v>Gospel of Thomas 39</x:v>
+      </x:c>
+      <x:c r="C24" s="83" t="str">
+        <x:v>The saying criticizes authorities who prevent entry to knowledge.</x:v>
+      </x:c>
+      <x:c r="D24" s="83" t="str">
+        <x:v>Thomas and formation</x:v>
+      </x:c>
+      <x:c r="E24" s="83" t="str">
+        <x:v>A shared criticism does not settle literary direction or the identity of a displaced priestly institution.</x:v>
+      </x:c>
+      <x:c r="F24" s="83" t="str">
+        <x:v>Gospel of Thomas, translation by Stephen Patterson and Marvin Meyer</x:v>
+      </x:c>
+      <x:c r="G24" s="83" t="str">
+        <x:v>Translation consulted for sayings 1, 3, 12, 13, 39 and 108. The edition uses brief paraphrases and links, not a reproduction of the translation. Translation credit is distinct from an acknowledged influence in the author's older conversations.</x:v>
+      </x:c>
+      <x:c r="H24" s="83" t="str">
+        <x:v>https://www.earlychristianwritings.com/text/thomas-scholars.html</x:v>
+      </x:c>
+      <x:c r="I24" s="83" t="str">
+        <x:v>thomas-coptic / jt-thomas-keys</x:v>
+      </x:c>
+      <x:c r="J24" s="83" t="str">
+        <x:v>Compare the operation of gatekeeping with Luke and proposed historical carriers.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="25" ht="120" customHeight="1">
+      <x:c r="A25" s="83" t="str">
+        <x:v>Blocked access to knowledge in Luke</x:v>
+      </x:c>
+      <x:c r="B25" s="83" t="str">
+        <x:v>Luke 11:52</x:v>
+      </x:c>
+      <x:c r="C25" s="83" t="str">
+        <x:v>A related accusation concerns experts who obstruct entry.</x:v>
+      </x:c>
+      <x:c r="D25" s="83" t="str">
+        <x:v>Thomas and formation</x:v>
+      </x:c>
+      <x:c r="E25" s="83" t="str">
+        <x:v>The relationship to Thomas can have more than one explanation.</x:v>
+      </x:c>
+      <x:c r="F25" s="83" t="str">
+        <x:v>Luke 11:52, World English Bible</x:v>
+      </x:c>
+      <x:c r="G25" s="83" t="str">
+        <x:v>Primary translated passage for the criticism of obstructed access to knowledge. A thematic and functional comparison with Thomas 39, not a demonstrated direction of literary dependence.</x:v>
+      </x:c>
+      <x:c r="H25" s="83" t="str">
+        <x:v>https://ebible.org/engwebp/LUK11.htm</x:v>
+      </x:c>
+      <x:c r="I25" s="83" t="str">
+        <x:v>luke / jt-luke-keys</x:v>
+      </x:c>
+      <x:c r="J25" s="83" t="str">
+        <x:v>Compare shared tradition, dependence and separate adaptation before selecting a transmission route.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="26" ht="120" customHeight="1">
+      <x:c r="A26" s="83" t="str">
+        <x:v>Non-material brotherhood in a James revelation</x:v>
+      </x:c>
+      <x:c r="B26" s="83" t="str">
+        <x:v>First Apocalypse of James, opening exchange</x:v>
+      </x:c>
+      <x:c r="C26" s="83" t="str">
+        <x:v>The opening explicitly distinguishes its brother language from material kinship.</x:v>
+      </x:c>
+      <x:c r="D26" s="83" t="str">
+        <x:v>Thomas and formation</x:v>
+      </x:c>
+      <x:c r="E26" s="83" t="str">
+        <x:v>This is a different text and setting from Galatians; direct page retrieval was unavailable and the opening was consulted through indexed translation.</x:v>
+      </x:c>
+      <x:c r="F26" s="83" t="str">
+        <x:v>First Apocalypse of James, William R. Schoedel translation</x:v>
+      </x:c>
+      <x:c r="G26" s="83" t="str">
+        <x:v>Consulted the opening distinction between material and spiritual brotherhood through the indexed translation. Direct page retrieval was unavailable during this intake. This is not a full-text review or a new Greek/Coptic collation.</x:v>
+      </x:c>
+      <x:c r="H26" s="83" t="str">
+        <x:v>https://www.gnosis.org/naghamm/1ja.html</x:v>
+      </x:c>
+      <x:c r="I26" s="83" t="str">
+        <x:v>first-apocalypse-james / jt-spiritual-brother</x:v>
+      </x:c>
+      <x:c r="J26" s="83" t="str">
+        <x:v>Test the meaning of each relational claim rather than moving a definition unchanged between genres.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="27" ht="120" customHeight="1">
+      <x:c r="A27" s="83" t="str">
+        <x:v>The actual coverage of partial Greek witnesses</x:v>
+      </x:c>
+      <x:c r="B27" s="83" t="str">
+        <x:v>Published extract, description of P.Oxy. 1 and P.Oxy. 655</x:v>
+      </x:c>
+      <x:c r="C27" s="83" t="str">
+        <x:v>The extract specifies partial saying coverage rather than a complete Greek collection.</x:v>
+      </x:c>
+      <x:c r="D27" s="83" t="str">
+        <x:v>Textual witnesses</x:v>
+      </x:c>
+      <x:c r="E27" s="83" t="str">
+        <x:v>The full article, line-41 proposal and manuscript images were not reviewed here.</x:v>
+      </x:c>
+      <x:c r="F27" s="83" t="str">
+        <x:v>Simon Gathercole, A Proposed Rereading of P.Oxy. 654 line 41 (Gos. Thom. 7), 2006</x:v>
+      </x:c>
+      <x:c r="G27" s="83" t="str">
+        <x:v>Consulted the Cambridge-published extract describing the partial Greek Thomas witnesses P.Oxy. 1 and P.Oxy. 655. The full article and proposed line-41 rereading were not reviewed; its witness description does not date the complete Coptic collection.</x:v>
+      </x:c>
+      <x:c r="H27" s="83" t="str">
+        <x:v>https://doi.org/10.1017/S0017816006001283</x:v>
+      </x:c>
+      <x:c r="I27" s="83" t="str">
+        <x:v>gathercole-2006 / jt-greek-thomas</x:v>
+      </x:c>
+      <x:c r="J27" s="83" t="str">
+        <x:v>Collate the witness containing each relevant saying before using a copy date for an entire collection.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="28" ht="120" customHeight="1">
+      <x:c r="A28" s="83" t="str">
+        <x:v>A copied James revelation and proposed educational use</x:v>
+      </x:c>
+      <x:c r="B28" s="83" t="str">
+        <x:v>University of Texas announcement, November 29, 2017</x:v>
+      </x:c>
+      <x:c r="C28" s="83" t="str">
+        <x:v>The researchers report fifth/sixth-century Greek fragments and infer educational use from syllabic divisions.</x:v>
+      </x:c>
+      <x:c r="D28" s="83" t="str">
+        <x:v>Textual witnesses</x:v>
+      </x:c>
+      <x:c r="E28" s="83" t="str">
+        <x:v>This is a reported First Apocalypse of James witness, not Thomas or a genealogical record; image rights remain with the named owner.</x:v>
+      </x:c>
+      <x:c r="F28" s="83" t="str">
+        <x:v>University of Texas, Smith and Landau report Greek First Apocalypse of James fragments, 2017</x:v>
+      </x:c>
+      <x:c r="G28" s="83" t="str">
+        <x:v>Institutional report of the researchers' discovery, published November 29, 2017. Fifth/sixth-century dating and possible educational use are reported interpretations. The later critical edition and physical fragments were not independently inspected. The report assigns fragment and image rights to the Egypt Exploration Society.</x:v>
+      </x:c>
+      <x:c r="H28" s="83" t="str">
+        <x:v>https://news.utexas.edu/2017/11/29/ut-austin-professors-discover-copy-of-jesus-secret-teaching/</x:v>
+      </x:c>
+      <x:c r="I28" s="83" t="str">
+        <x:v>ut-james-2017 / jt-greek-james</x:v>
+      </x:c>
+      <x:c r="J28" s="83" t="str">
+        <x:v>Review the critical publication and competing explanations of the scribal format.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="29" ht="120" customHeight="1">
+      <x:c r="A29" s="83" t="str">
+        <x:v>An earlier James and visionary-reading comparison</x:v>
+      </x:c>
+      <x:c r="B29" s="83" t="str">
+        <x:v>The Gospel of Thomas and the Hermeneutics of Vision, 2002 essay</x:v>
+      </x:c>
+      <x:c r="C29" s="83" t="str">
+        <x:v>Owens connects James, apocalyptic inheritance and transformation of the interpreter.</x:v>
+      </x:c>
+      <x:c r="D29" s="83" t="str">
+        <x:v>Interpretive research</x:v>
+      </x:c>
+      <x:c r="E29" s="83" t="str">
+        <x:v>The comparison is not a demonstrated genealogy or a documented influence on the older conversations.</x:v>
+      </x:c>
+      <x:c r="F29" s="83" t="str">
+        <x:v>Lance S. Owens, The Gospel of Thomas and the Hermeneutics of Vision, 2002</x:v>
+      </x:c>
+      <x:c r="G29" s="83" t="str">
+        <x:v>Earlier interpretive essay, copyright 2002, consulted through indexed text. Credits the James/apocalyptic/transformative-reading comparison without adopting all historical assertions or claiming a demonstrated chain to Kabbalah. This is a newly consulted comparison, not a documented personal influence on the older conversations.</x:v>
+      </x:c>
+      <x:c r="H29" s="83" t="str">
+        <x:v>https://www.gnosis.org/naghamm/gth_hermen.htm</x:v>
+      </x:c>
+      <x:c r="I29" s="83" t="str">
+        <x:v>owens-2002 / jt-owens-vision</x:v>
+      </x:c>
+      <x:c r="J29" s="83" t="str">
+        <x:v>Credit the preceding interpretation and distinguish the additional earlier-founder chronological claim.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="30" ht="120" customHeight="1">
+      <x:c r="A30" s="83" t="str">
+        <x:v>Daniel 9:24-27</x:v>
+      </x:c>
+      <x:c r="B30" s="83" t="str">
+        <x:v>Daniel 9:24-27</x:v>
+      </x:c>
+      <x:c r="C30" s="83" t="str">
+        <x:v>Seven weeks, 62 weeks and a final week require explicit event assignments.</x:v>
+      </x:c>
+      <x:c r="D30" s="83" t="str">
+        <x:v>Priesthood and prophetic time</x:v>
+      </x:c>
+      <x:c r="E30" s="83" t="str">
+        <x:v>A numerical sequence alone does not identify its persons or choose a modern calendar anchor.</x:v>
+      </x:c>
+      <x:c r="F30" s="83" t="str">
+        <x:v>Daniel 9, World English Bible</x:v>
+      </x:c>
+      <x:c r="G30" s="83" t="str">
+        <x:v>Primary translated chapter consulted, especially verses 2, 15, 17 and 24-27. Exodus, sanctuary, desolation and restoration remain separate from any proposed absolute-year calculation.</x:v>
+      </x:c>
+      <x:c r="H30" s="83" t="str">
+        <x:v>https://ebible.org/engwebp/DAN09.htm</x:v>
+      </x:c>
+      <x:c r="I30" s="83" t="str">
+        <x:v>daniel / pt-daniel-order</x:v>
+      </x:c>
+      <x:c r="J30" s="83" t="str">
+        <x:v>State the beginning event and which anointed figure belongs to each interval.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="31" ht="120" customHeight="1">
+      <x:c r="A31" s="83" t="str">
+        <x:v>CD 1:3-11, as discussed in Collins section J</x:v>
+      </x:c>
+      <x:c r="B31" s="83" t="str">
+        <x:v>CD 1:3-11, as discussed in Collins section J</x:v>
+      </x:c>
+      <x:c r="C31" s="83" t="str">
+        <x:v>390 years followed by 20 precede the Teacher's appearance in the discussed chronology.</x:v>
+      </x:c>
+      <x:c r="D31" s="83" t="str">
+        <x:v>Priesthood and prophetic time</x:v>
+      </x:c>
+      <x:c r="E31" s="83" t="str">
+        <x:v>A chosen 586 BCE anchor yields an illustrative 176 BCE appearance, not a date inscribed in the text.</x:v>
+      </x:c>
+      <x:c r="F31" s="83" t="str">
+        <x:v>John J. Collins, The Dead Sea Scrolls (Anchor Bible Dictionary, 1992)</x:v>
+      </x:c>
+      <x:c r="G31" s="83" t="str">
+        <x:v>Sections C and J of the full online reproduction consulted for CD 1, CD 20:15, and household rules at CD 7:6-7. The 40-year Teacher career is a reconstructed interval. This is a dated scholarly interpretation, not a new Hebrew collation or current manuscript inventory.</x:v>
+      </x:c>
+      <x:c r="H31" s="83" t="str">
+        <x:v>https://cojs.org/the_dead_sea_scrolls-_john_j-_collins-_anchor_bible_dictionary_-ed-_david_noel_freedman-_doubleday-_ny-_1992-_vol-2-_p-85-101/</x:v>
+      </x:c>
+      <x:c r="I31" s="83" t="str">
+        <x:v>collins-damascus / pt-cd-appearance</x:v>
+      </x:c>
+      <x:c r="J31" s="83" t="str">
+        <x:v>Collate the Hebrew witness and evaluate independent anchoring evidence.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="32" ht="120" customHeight="1">
+      <x:c r="A32" s="83" t="str">
+        <x:v>CD 20:15 and Collins section J</x:v>
+      </x:c>
+      <x:c r="B32" s="83" t="str">
+        <x:v>CD 20:15 and Collins section J</x:v>
+      </x:c>
+      <x:c r="C32" s="83" t="str">
+        <x:v>The reconstructed 40-year career completes 390 + 20 + 40 + 40 = 490.</x:v>
+      </x:c>
+      <x:c r="D32" s="83" t="str">
+        <x:v>Priesthood and prophetic time</x:v>
+      </x:c>
+      <x:c r="E32" s="83" t="str">
+        <x:v>The career interval is supplied; it must not be labeled as directly attested like the other intervals.</x:v>
+      </x:c>
+      <x:c r="F32" s="83" t="str">
+        <x:v>John J. Collins, The Dead Sea Scrolls (Anchor Bible Dictionary, 1992)</x:v>
+      </x:c>
+      <x:c r="G32" s="83" t="str">
+        <x:v>Sections C and J of the full online reproduction consulted for CD 1, CD 20:15, and household rules at CD 7:6-7. The 40-year Teacher career is a reconstructed interval. This is a dated scholarly interpretation, not a new Hebrew collation or current manuscript inventory.</x:v>
+      </x:c>
+      <x:c r="H32" s="83" t="str">
+        <x:v>https://cojs.org/the_dead_sea_scrolls-_john_j-_collins-_anchor_bible_dictionary_-ed-_david_noel_freedman-_doubleday-_ny-_1992-_vol-2-_p-85-101/</x:v>
+      </x:c>
+      <x:c r="I32" s="83" t="str">
+        <x:v>collins-damascus / pt-cd-career</x:v>
+      </x:c>
+      <x:c r="J32" s="83" t="str">
+        <x:v>Compare proposed career, office and generation interpretations before identifying a death.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="33" ht="120" customHeight="1">
+      <x:c r="A33" s="83" t="str">
+        <x:v>11Q13 II 6-7 in Williams's translation and discussion</x:v>
+      </x:c>
+      <x:c r="B33" s="83" t="str">
+        <x:v>11Q13 II 6-7 in Williams's translation and discussion</x:v>
+      </x:c>
+      <x:c r="C33" s="83" t="str">
+        <x:v>Williams adopts a reading placing liberation at the beginning of the cycle after ten jubilees.</x:v>
+      </x:c>
+      <x:c r="D33" s="83" t="str">
+        <x:v>Priesthood and prophetic time</x:v>
+      </x:c>
+      <x:c r="E33" s="83" t="str">
+        <x:v>The older tenth-jubilee reading remains a distinct restoration; neither fixes a Teacher identity or a BCE date.</x:v>
+      </x:c>
+      <x:c r="F33" s="83" t="str">
+        <x:v>Logan Williams (2023), Melchizedek, the Son of Man, and Eschatological Jubilee</x:v>
+      </x:c>
+      <x:c r="G33" s="83" t="str">
+        <x:v>Full-text HTML consulted, particularly the author's translation of 11Q13 II 2-9 and discussion of II 6 and 13. His active-agent reading is distinguished from the critical edition he disputes. The critical edition itself has not been collated in this pass. This is current editorial research, not a recovered author acknowledgment.</x:v>
+      </x:c>
+      <x:c r="H33" s="83" t="str">
+        <x:v>https://journals.sagepub.com/doi/10.1177/0142064X231191176</x:v>
+      </x:c>
+      <x:c r="I33" s="83" t="str">
+        <x:v>williams-melchizedek / pt-jubilee</x:v>
+      </x:c>
+      <x:c r="J33" s="83" t="str">
+        <x:v>Independently collate II 6-7 and II 18 against the critical edition and photographs.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="34" ht="120" customHeight="1">
+      <x:c r="A34" s="83" t="str">
+        <x:v>Published abstract, DOI 10.31743/vv.1935</x:v>
+      </x:c>
+      <x:c r="B34" s="83" t="str">
+        <x:v>Published abstract, DOI 10.31743/vv.1935</x:v>
+      </x:c>
+      <x:c r="C34" s="83" t="str">
+        <x:v>364-day and 365-day idealized units differ by 490 days across 490 years.</x:v>
+      </x:c>
+      <x:c r="D34" s="83" t="str">
+        <x:v>Priesthood and prophetic time</x:v>
+      </x:c>
+      <x:c r="E34" s="83" t="str">
+        <x:v>This is not a model of practical intercalation and cannot alone shift a chronology by a century.</x:v>
+      </x:c>
+      <x:c r="F34" s="83" t="str">
+        <x:v>Michal Jaroslaw Klukowski, The Tradition of the 364-Day Year in Second Temple Period Judaism</x:v>
+      </x:c>
+      <x:c r="G34" s="83" t="str">
+        <x:v>Published scholarly abstract consulted for the 364-day schematic-year tradition and its relationship to calendrical texts. No claim of full-paper review, a settled origin, or a proved practical intercalation scheme is made.</x:v>
+      </x:c>
+      <x:c r="H34" s="83" t="str">
+        <x:v>https://czasopisma.kul.pl/index.php/vv/article/view/1935</x:v>
+      </x:c>
+      <x:c r="I34" s="83" t="str">
+        <x:v>priests-calendar / pt-calendar</x:v>
+      </x:c>
+      <x:c r="J34" s="83" t="str">
+        <x:v>Distinguish calendar operation from the count's chosen historical starting event.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="35" ht="120" customHeight="1">
+      <x:c r="A35" s="83" t="str">
+        <x:v>Antiquities 13.3.1-3</x:v>
+      </x:c>
+      <x:c r="B35" s="83" t="str">
+        <x:v>Antiquities 13.3.1-3</x:v>
+      </x:c>
+      <x:c r="C35" s="83" t="str">
+        <x:v>The account supplies royal permission, priests and Levites, and a scriptural argument for a sanctuary in Egypt.</x:v>
+      </x:c>
+      <x:c r="D35" s="83" t="str">
+        <x:v>Priesthood and prophetic time</x:v>
+      </x:c>
+      <x:c r="E35" s="83" t="str">
+        <x:v>Reported correspondence is not an independently inspected original royal document.</x:v>
+      </x:c>
+      <x:c r="F35" s="83" t="str">
+        <x:v>Josephus, Antiquities 13.3.1-3, 13.10.4 and 13.13.2, Whiston translation</x:v>
+      </x:c>
+      <x:c r="G35" s="83" t="str">
+        <x:v>Primary translated passages consulted for the sanctuary, royal petition and permission, Onias's sons Chelcias and Ananias, and Ananias's counsel concerning Alexander. Strabo is encountered through Josephus's quotation, not as an independently inspected document. These relations do not establish subsequent Teacher or Gnostic transmission.</x:v>
+      </x:c>
+      <x:c r="H35" s="83" t="str">
+        <x:v>https://penelope.uchicago.edu/josephus/ant-13.html</x:v>
+      </x:c>
+      <x:c r="I35" s="83" t="str">
+        <x:v>josephus-antiquities / pt-sanctuary</x:v>
+      </x:c>
+      <x:c r="J35" s="83" t="str">
+        <x:v>Compare the Greek text, the identity of the founder and competing foundation dates.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="36" ht="120" customHeight="1">
+      <x:c r="A36" s="83" t="str">
+        <x:v>Antiquities 13.10.4 and 13.13.2</x:v>
+      </x:c>
+      <x:c r="B36" s="83" t="str">
+        <x:v>Antiquities 13.10.4 and 13.13.2</x:v>
+      </x:c>
+      <x:c r="C36" s="83" t="str">
+        <x:v>Chelcias and Ananias are identified as sons of the founder; Ananias defends Alexander against a proposed dispossession.</x:v>
+      </x:c>
+      <x:c r="D36" s="83" t="str">
+        <x:v>Priesthood and prophetic time</x:v>
+      </x:c>
+      <x:c r="E36" s="83" t="str">
+        <x:v>This supplies candidate carriers and contact, not proof of Essene affiliation or Thomas transmission.</x:v>
+      </x:c>
+      <x:c r="F36" s="83" t="str">
+        <x:v>Josephus, Antiquities 13.3.1-3, 13.10.4 and 13.13.2, Whiston translation</x:v>
+      </x:c>
+      <x:c r="G36" s="83" t="str">
+        <x:v>Primary translated passages consulted for the sanctuary, royal petition and permission, Onias's sons Chelcias and Ananias, and Ananias's counsel concerning Alexander. Strabo is encountered through Josephus's quotation, not as an independently inspected document. These relations do not establish subsequent Teacher or Gnostic transmission.</x:v>
+      </x:c>
+      <x:c r="H36" s="83" t="str">
+        <x:v>https://penelope.uchicago.edu/josephus/ant-13.html</x:v>
+      </x:c>
+      <x:c r="I36" s="83" t="str">
+        <x:v>josephus-antiquities / pt-sons</x:v>
+      </x:c>
+      <x:c r="J36" s="83" t="str">
+        <x:v>Trace the family and institutional relations in independently supported evidence.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="37" ht="120" customHeight="1">
+      <x:c r="A37" s="83" t="str">
+        <x:v>War 7.10.2-3 compared with Antiquities 13.3.1-3</x:v>
+      </x:c>
+      <x:c r="B37" s="83" t="str">
+        <x:v>War 7.10.2-3 compared with Antiquities 13.3.1-3</x:v>
+      </x:c>
+      <x:c r="C37" s="83" t="str">
+        <x:v>Parentage and architectural particulars differ across the two accounts.</x:v>
+      </x:c>
+      <x:c r="D37" s="83" t="str">
+        <x:v>Priesthood and prophetic time</x:v>
+      </x:c>
+      <x:c r="E37" s="83" t="str">
+        <x:v>Do not silently turn son of Simon and son of Onias into one agreed identification.</x:v>
+      </x:c>
+      <x:c r="F37" s="83" t="str">
+        <x:v>Josephus, War 7.10.2-4, William Whiston translation</x:v>
+      </x:c>
+      <x:c r="G37" s="83" t="str">
+        <x:v>Primary translated narrative consulted for the Onias sanctuary, different parentage and architectural description, support and closure under Lupus and Paulinus, and the transmitted 343-year duration. Editorial bracketed dates and Whiston notes are not words of the ancient narrative.</x:v>
+      </x:c>
+      <x:c r="H37" s="83" t="str">
+        <x:v>https://penelope.uchicago.edu/josephus/war-7.html</x:v>
+      </x:c>
+      <x:c r="I37" s="83" t="str">
+        <x:v>josephus-war / pt-conflict</x:v>
+      </x:c>
+      <x:c r="J37" s="83" t="str">
+        <x:v>Record variant readings, authorial development and competing historical explanations.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="38" ht="120" customHeight="1">
+      <x:c r="A38" s="83" t="str">
+        <x:v>War 7.10.4</x:v>
+      </x:c>
+      <x:c r="B38" s="83" t="str">
+        <x:v>War 7.10.4</x:v>
+      </x:c>
+      <x:c r="C38" s="83" t="str">
+        <x:v>Lupus and Paulinus restrict the sanctuary; the transmitted duration is 343 years.</x:v>
+      </x:c>
+      <x:c r="D38" s="83" t="str">
+        <x:v>Priesthood and prophetic time</x:v>
+      </x:c>
+      <x:c r="E38" s="83" t="str">
+        <x:v>No precise foundation or closure date is adopted from this inconsistent duration.</x:v>
+      </x:c>
+      <x:c r="F38" s="83" t="str">
+        <x:v>Josephus, War 7.10.2-4, William Whiston translation</x:v>
+      </x:c>
+      <x:c r="G38" s="83" t="str">
+        <x:v>Primary translated narrative consulted for the Onias sanctuary, different parentage and architectural description, support and closure under Lupus and Paulinus, and the transmitted 343-year duration. Editorial bracketed dates and Whiston notes are not words of the ancient narrative.</x:v>
+      </x:c>
+      <x:c r="H38" s="83" t="str">
+        <x:v>https://penelope.uchicago.edu/josephus/war-7.html</x:v>
+      </x:c>
+      <x:c r="I38" s="83" t="str">
+        <x:v>josephus-war / pt-closure</x:v>
+      </x:c>
+      <x:c r="J38" s="83" t="str">
+        <x:v>Investigate contacts before closure and possible dispersed institutions afterward.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="39" ht="120" customHeight="1">
+      <x:c r="A39" s="83" t="str">
+        <x:v>War 2.8.13; compare CD 7:6-7 through Collins</x:v>
+      </x:c>
+      <x:c r="B39" s="83" t="str">
+        <x:v>War 2.8.13; compare CD 7:6-7 through Collins</x:v>
+      </x:c>
+      <x:c r="C39" s="83" t="str">
+        <x:v>Josephus describes a marrying Essene order concerned with succession.</x:v>
+      </x:c>
+      <x:c r="D39" s="83" t="str">
+        <x:v>Priesthood and prophetic time</x:v>
+      </x:c>
+      <x:c r="E39" s="83" t="str">
+        <x:v>A wider household population does not establish the proposed demographic split or identify every community.</x:v>
+      </x:c>
+      <x:c r="F39" s="83" t="str">
+        <x:v>Josephus, War 2.8.13, William Whiston translation</x:v>
+      </x:c>
+      <x:c r="G39" s="83" t="str">
+        <x:v>Primary translated passage consulted for the marrying Essene order and its concern with succession. It is not a roster of the households or branches proposed in this reconstruction.</x:v>
+      </x:c>
+      <x:c r="H39" s="83" t="str">
+        <x:v>https://penelope.uchicago.edu/josephus/war-2.html</x:v>
+      </x:c>
+      <x:c r="I39" s="83" t="str">
+        <x:v>josephus-war / pt-households</x:v>
+      </x:c>
+      <x:c r="J39" s="83" t="str">
+        <x:v>Compare household rules, actual names and institutional practice without a uniform celibate stereotype.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="40" ht="120" customHeight="1">
+      <x:c r="A40" s="83" t="str">
+        <x:v>Second Maccabees 4:33-38</x:v>
+      </x:c>
+      <x:c r="B40" s="83" t="str">
+        <x:v>Second Maccabees 4:33-38</x:v>
+      </x:c>
+      <x:c r="C40" s="83" t="str">
+        <x:v>The passage identifies relations around a priestly murder involving Onias and Andronicus.</x:v>
+      </x:c>
+      <x:c r="D40" s="83" t="str">
+        <x:v>Priesthood and prophetic time</x:v>
+      </x:c>
+      <x:c r="E40" s="83" t="str">
+        <x:v>The John-the-Baptist identification and a 20-year transition are additional claims.</x:v>
+      </x:c>
+      <x:c r="F40" s="83" t="str">
+        <x:v>Second Maccabees 4:33-38, USCCB translation</x:v>
+      </x:c>
+      <x:c r="G40" s="83" t="str">
+        <x:v>Primary translated passage consulted for the death of Onias, the roles of Andronicus and Menelaus, and the king's response. It does not itself identify John the Baptist or a 20-year interval to the Teacher.</x:v>
+      </x:c>
+      <x:c r="H40" s="83" t="str">
+        <x:v>https://bible.usccb.org/bible/2maccabees/4</x:v>
+      </x:c>
+      <x:c r="I40" s="83" t="str">
+        <x:v>priests-macc4 / pt-predecessor</x:v>
+      </x:c>
+      <x:c r="J40" s="83" t="str">
+        <x:v>Compare narrative sequence and historical carriers, not merely a shared execution motif.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="41" ht="120" customHeight="1">
+      <x:c r="A41" s="83" t="str">
+        <x:v>Published abstract, Scripta Classica Israelica 16 (1997), 47-70</x:v>
+      </x:c>
+      <x:c r="B41" s="83" t="str">
+        <x:v>Published abstract, Scripta Classica Israelica 16 (1997), 47-70</x:v>
+      </x:c>
+      <x:c r="C41" s="83" t="str">
+        <x:v>Gruen proposes mutual support rather than a simply rival sanctuary model.</x:v>
+      </x:c>
+      <x:c r="D41" s="83" t="str">
+        <x:v>Priesthood and prophetic time</x:v>
+      </x:c>
+      <x:c r="E41" s="83" t="str">
+        <x:v>Full-paper review and endorsement of the broader branch genealogy are not claimed.</x:v>
+      </x:c>
+      <x:c r="F41" s="83" t="str">
+        <x:v>Erich S. Gruen, The Origins and Objectives of Onias' Temple (1997)</x:v>
+      </x:c>
+      <x:c r="G41" s="83" t="str">
+        <x:v>Published abstract consulted. It challenges the conventional rival-temple account and proposes mutual support between Jerusalem and Leontopolis while noting problems in Josephus. The full article and its critical apparatus were not independently reviewed in this pass; publication is 1997, not the website upload date.</x:v>
+      </x:c>
+      <x:c r="H41" s="83" t="str">
+        <x:v>https://scriptaclassica.org/index.php/sci/article/view/4239</x:v>
+      </x:c>
+      <x:c r="I41" s="83" t="str">
+        <x:v>priests-gruen / pt-cooperation</x:v>
+      </x:c>
+      <x:c r="J41" s="83" t="str">
+        <x:v>Consult the full critical discussion and compare its argument with the actual Josephus passages.</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -20074,7 +21273,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc5b7725588224b17"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R16d8bf625b794cf7"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -20092,32 +21291,32 @@
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="36" customHeight="1">
-      <x:c r="A1" s="5" t="str">
+      <x:c r="A1" s="69" t="str">
         <x:v>Theology | Credit and source lineage</x:v>
       </x:c>
-      <x:c r="B1" s="5"/>
-      <x:c r="C1" s="5"/>
-      <x:c r="D1" s="5"/>
-      <x:c r="E1" s="5"/>
-      <x:c r="F1" s="5"/>
+      <x:c r="B1" s="69"/>
+      <x:c r="C1" s="69"/>
+      <x:c r="D1" s="69"/>
+      <x:c r="E1" s="69"/>
+      <x:c r="F1" s="69"/>
     </x:row>
     <x:row r="2" ht="22" customHeight="1">
-      <x:c r="A2" s="10" t="str">
+      <x:c r="A2" s="71" t="str">
         <x:v>An author acknowledgment, an edition-used translation, an AI-introduced lead and an independent scholarly argument are not interchangeable.</x:v>
       </x:c>
-      <x:c r="B2" s="10"/>
-      <x:c r="C2" s="10"/>
-      <x:c r="D2" s="10"/>
-      <x:c r="E2" s="10"/>
-      <x:c r="F2" s="10"/>
+      <x:c r="B2" s="71"/>
+      <x:c r="C2" s="71"/>
+      <x:c r="D2" s="71"/>
+      <x:c r="E2" s="71"/>
+      <x:c r="F2" s="71"/>
     </x:row>
     <x:row r="3" ht="22" customHeight="1">
-      <x:c r="A3" s="10"/>
-      <x:c r="B3" s="10"/>
-      <x:c r="C3" s="10"/>
-      <x:c r="D3" s="10"/>
-      <x:c r="E3" s="10"/>
-      <x:c r="F3" s="10"/>
+      <x:c r="A3" s="71"/>
+      <x:c r="B3" s="71"/>
+      <x:c r="C3" s="71"/>
+      <x:c r="D3" s="71"/>
+      <x:c r="E3" s="71"/>
+      <x:c r="F3" s="71"/>
     </x:row>
     <x:row r="4">
       <x:c r="A4" s="2"/>
@@ -20128,8 +21327,8 @@
       <x:c r="F4" s="2"/>
     </x:row>
     <x:row r="5" ht="20" customHeight="1">
-      <x:c r="A5" s="14" t="str">
-        <x:v>Snapshot 2026-09-05 | 2026.09.05-atlas-1 | Shared plan: theology-wiki/editorial/roadmap.json</x:v>
+      <x:c r="A5" s="72" t="str">
+        <x:v>Content edition: 2026.09.06-james-transmission-1</x:v>
       </x:c>
       <x:c r="B5" s="14"/>
       <x:c r="C5" s="14"/>
@@ -20269,6 +21468,26 @@
       <x:c r="E12" s="23" t="str"/>
       <x:c r="F12" s="23" t="str">
         <x:v>https://journals.sagepub.com/doi/10.1177/0142064X231191176</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="13" ht="120" customHeight="1">
+      <x:c r="A13" s="84" t="str">
+        <x:v>Lance S. Owens</x:v>
+      </x:c>
+      <x:c r="B13" s="84" t="str">
+        <x:v>Newly consulted earlier interpretation</x:v>
+      </x:c>
+      <x:c r="C13" s="84" t="str">
+        <x:v>The 2002 essay already connects Thomas, James, apocalyptic inheritance and transformation of the interpreter.</x:v>
+      </x:c>
+      <x:c r="D13" s="84" t="str">
+        <x:v>Not a recovered personal acknowledgment from older conversations; no claim that the essay establishes the proposed earlier-founder chronology or a complete transmission chain to Kabbalah.</x:v>
+      </x:c>
+      <x:c r="E13" s="84" t="str">
+        <x:v>Newly consulted; no original acknowledgment claimed</x:v>
+      </x:c>
+      <x:c r="F13" s="84" t="str">
+        <x:v>https://www.gnosis.org/naghamm/gth_hermen.htm</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -20279,7 +21498,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7741f83ca59f4f82"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rcf2b919920d64ddf"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -20296,29 +21515,29 @@
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="36" customHeight="1">
-      <x:c r="A1" s="5" t="str">
+      <x:c r="A1" s="69" t="str">
         <x:v>Theology | Readiness is evidence, not word count</x:v>
       </x:c>
-      <x:c r="B1" s="5"/>
-      <x:c r="C1" s="5"/>
-      <x:c r="D1" s="5"/>
-      <x:c r="E1" s="5"/>
+      <x:c r="B1" s="69"/>
+      <x:c r="C1" s="69"/>
+      <x:c r="D1" s="69"/>
+      <x:c r="E1" s="69"/>
     </x:row>
     <x:row r="2" ht="22" customHeight="1">
-      <x:c r="A2" s="10" t="str">
+      <x:c r="A2" s="71" t="str">
         <x:v>These are whole-manuscript gates. A completed tool, article draft or word-count target does not pass them automatically.</x:v>
       </x:c>
-      <x:c r="B2" s="10"/>
-      <x:c r="C2" s="10"/>
-      <x:c r="D2" s="10"/>
-      <x:c r="E2" s="10"/>
+      <x:c r="B2" s="71"/>
+      <x:c r="C2" s="71"/>
+      <x:c r="D2" s="71"/>
+      <x:c r="E2" s="71"/>
     </x:row>
     <x:row r="3" ht="22" customHeight="1">
-      <x:c r="A3" s="10"/>
-      <x:c r="B3" s="10"/>
-      <x:c r="C3" s="10"/>
-      <x:c r="D3" s="10"/>
-      <x:c r="E3" s="10"/>
+      <x:c r="A3" s="71"/>
+      <x:c r="B3" s="71"/>
+      <x:c r="C3" s="71"/>
+      <x:c r="D3" s="71"/>
+      <x:c r="E3" s="71"/>
     </x:row>
     <x:row r="4">
       <x:c r="A4" s="2"/>
@@ -20328,8 +21547,8 @@
       <x:c r="E4" s="2"/>
     </x:row>
     <x:row r="5" ht="20" customHeight="1">
-      <x:c r="A5" s="14" t="str">
-        <x:v>Snapshot 2026-09-05 | 2026.09.05-atlas-1 | Shared plan: theology-wiki/editorial/roadmap.json</x:v>
+      <x:c r="A5" s="72" t="str">
+        <x:v>Content edition: 2026.09.06-james-transmission-1</x:v>
       </x:c>
       <x:c r="B5" s="14"/>
       <x:c r="C5" s="14"/>
@@ -20485,7 +21704,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R491a4979174646a7"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3253eb8a136c4b7d"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -20499,28 +21718,28 @@
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="36" customHeight="1">
-      <x:c r="A1" s="5" t="str">
+      <x:c r="A1" s="69" t="str">
         <x:v>Theology | How to use and maintain this plan</x:v>
       </x:c>
-      <x:c r="B1" s="5"/>
+      <x:c r="B1" s="69"/>
     </x:row>
     <x:row r="2" ht="22" customHeight="1">
-      <x:c r="A2" s="10" t="str">
+      <x:c r="A2" s="71" t="str">
         <x:v>Read the limits before interpreting the dashboard. Source-backed planning and author approval are deliberately separate.</x:v>
       </x:c>
-      <x:c r="B2" s="10"/>
+      <x:c r="B2" s="71"/>
     </x:row>
     <x:row r="3" ht="22" customHeight="1">
-      <x:c r="A3" s="10"/>
-      <x:c r="B3" s="10"/>
+      <x:c r="A3" s="71"/>
+      <x:c r="B3" s="71"/>
     </x:row>
     <x:row r="4">
       <x:c r="A4" s="2"/>
       <x:c r="B4" s="2"/>
     </x:row>
     <x:row r="5" ht="20" customHeight="1">
-      <x:c r="A5" s="14" t="str">
-        <x:v>Snapshot 2026-09-05 | 2026.09.05-atlas-1 | Shared plan: theology-wiki/editorial/roadmap.json</x:v>
+      <x:c r="A5" s="72" t="str">
+        <x:v>Content edition: 2026.09.06-james-transmission-1</x:v>
       </x:c>
       <x:c r="B5" s="14"/>
     </x:row>
@@ -20625,7 +21844,7 @@
         <x:v>Next writing pass</x:v>
       </x:c>
       <x:c r="B18" s="23" t="str">
-        <x:v>Review the Daniel and Onias studies, then pursue the precise critical editions and historical intermediates recorded in each task. New comparison work does not confer author approval or validate an entire reconstruction.</x:v>
+        <x:v>Collate Greek and Coptic witnesses; develop the Jamesian institutional route. Use the evidence workbench to distinguish shared channels, contributions and unresolved questions.</x:v>
       </x:c>
     </x:row>
     <x:row r="19" ht="64" customHeight="1">
@@ -20649,7 +21868,7 @@
         <x:v>Connected foundations refresh</x:v>
       </x:c>
       <x:c r="B21" s="23" t="str">
-        <x:v>2026-09-06. The book routes now include computational divine immanence and flood inheritance. Coherence and formal-comparison tasks are Draft; author approval and independent argument checks remain open.</x:v>
+        <x:v>2026.09.06-james-transmission-1. Two new full studies, 30 claim-level records, and ten new museum stops. Current shared statuses remain bounded deliverables, not author approval.</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -20660,7 +21879,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R92c699935969427a"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R07a578b40ce74458"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>